<commit_message>
Change rule calculate R_ref_simple
</commit_message>
<xml_diff>
--- a/outputs/bond_results_tier2_oas.xlsx
+++ b/outputs/bond_results_tier2_oas.xlsx
@@ -606,13 +606,13 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <v>99.39118065167645</v>
+        <v>78.71632465393753</v>
       </c>
       <c r="C2">
-        <v>99.4175104210877</v>
+        <v>78.61800974190142</v>
       </c>
       <c r="D2">
-        <v>-0.02632976941124809</v>
+        <v>0.0983149120361162</v>
       </c>
       <c r="E2" t="s">
         <v>63</v>
@@ -623,13 +623,13 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>91.71152036401712</v>
+        <v>62.55112430626606</v>
       </c>
       <c r="C3">
-        <v>91.64550210775943</v>
+        <v>62.47574730567867</v>
       </c>
       <c r="D3">
-        <v>0.06601825625769209</v>
+        <v>0.0753770005873875</v>
       </c>
       <c r="E3" t="s">
         <v>64</v>
@@ -640,13 +640,13 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>107.6790532548355</v>
+        <v>99.88602801317066</v>
       </c>
       <c r="C4">
-        <v>109.6498382311094</v>
+        <v>99.9094013158531</v>
       </c>
       <c r="D4">
-        <v>-1.970784976273961</v>
+        <v>-0.02337330268244386</v>
       </c>
       <c r="E4" t="s">
         <v>65</v>
@@ -657,13 +657,13 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>97.35349500005347</v>
+        <v>72.81859329746192</v>
       </c>
       <c r="C5">
-        <v>97.2916801669969</v>
+        <v>72.72898903587709</v>
       </c>
       <c r="D5">
-        <v>0.06181483305657309</v>
+        <v>0.08960426158482448</v>
       </c>
       <c r="E5" t="s">
         <v>66</v>
@@ -674,13 +674,13 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>99.46769251326324</v>
+        <v>81.32835344913367</v>
       </c>
       <c r="C6">
-        <v>100.6122239440398</v>
+        <v>81.22620470161775</v>
       </c>
       <c r="D6">
-        <v>-1.144531430776567</v>
+        <v>0.1021487475159262</v>
       </c>
       <c r="E6" t="s">
         <v>67</v>
@@ -691,13 +691,13 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>96.7405577127613</v>
+        <v>74.46635902185859</v>
       </c>
       <c r="C7">
-        <v>97.25698393741723</v>
+        <v>74.3737790519146</v>
       </c>
       <c r="D7">
-        <v>-0.5164262246559304</v>
+        <v>0.09257996994399775</v>
       </c>
       <c r="E7" t="s">
         <v>68</v>
@@ -708,13 +708,13 @@
         <v>5</v>
       </c>
       <c r="B8">
-        <v>101.866985126583</v>
+        <v>83.22752315091005</v>
       </c>
       <c r="C8">
-        <v>101.9373424554063</v>
+        <v>83.12311314704344</v>
       </c>
       <c r="D8">
-        <v>-0.07035732882329171</v>
+        <v>0.1044100038666045</v>
       </c>
       <c r="E8" t="s">
         <v>69</v>
@@ -725,13 +725,13 @@
         <v>6</v>
       </c>
       <c r="B9">
-        <v>104.4102654916629</v>
+        <v>86.92124127858565</v>
       </c>
       <c r="C9">
-        <v>104.2975535277135</v>
+        <v>86.82326312635855</v>
       </c>
       <c r="D9">
-        <v>0.1127119639494083</v>
+        <v>0.09797815222709971</v>
       </c>
       <c r="E9" t="s">
         <v>63</v>
@@ -742,13 +742,13 @@
         <v>6</v>
       </c>
       <c r="B10">
-        <v>104.0139088705514</v>
+        <v>75.01159072882399</v>
       </c>
       <c r="C10">
-        <v>103.9079239567337</v>
+        <v>74.92789141620285</v>
       </c>
       <c r="D10">
-        <v>0.1059849138177356</v>
+        <v>0.08369931262113539</v>
       </c>
       <c r="E10" t="s">
         <v>64</v>
@@ -759,13 +759,13 @@
         <v>6</v>
       </c>
       <c r="B11">
-        <v>105.6395785308202</v>
+        <v>100.8895759068823</v>
       </c>
       <c r="C11">
-        <v>105.5189273180302</v>
+        <v>100.7748317904294</v>
       </c>
       <c r="D11">
-        <v>0.1206512127900652</v>
+        <v>0.1147441164529397</v>
       </c>
       <c r="E11" t="s">
         <v>65</v>
@@ -776,13 +776,13 @@
         <v>6</v>
       </c>
       <c r="B12">
-        <v>102.7694033553193</v>
+        <v>85.96046271672296</v>
       </c>
       <c r="C12">
-        <v>102.656134878459</v>
+        <v>85.86372331766567</v>
       </c>
       <c r="D12">
-        <v>0.1132684768602843</v>
+        <v>0.09673939905728446</v>
       </c>
       <c r="E12" t="s">
         <v>66</v>
@@ -793,13 +793,13 @@
         <v>6</v>
       </c>
       <c r="B13">
-        <v>106.1835106747425</v>
+        <v>85.32664861938335</v>
       </c>
       <c r="C13">
-        <v>106.0725325691629</v>
+        <v>85.23049714258354</v>
       </c>
       <c r="D13">
-        <v>0.110978105579548</v>
+        <v>0.09615147679980396</v>
       </c>
       <c r="E13" t="s">
         <v>67</v>
@@ -810,13 +810,13 @@
         <v>6</v>
       </c>
       <c r="B14">
-        <v>105.9358623015307</v>
+        <v>80.98994465457615</v>
       </c>
       <c r="C14">
-        <v>105.8271920706346</v>
+        <v>80.89900034277123</v>
       </c>
       <c r="D14">
-        <v>0.108670230896152</v>
+        <v>0.09094431180491824</v>
       </c>
       <c r="E14" t="s">
         <v>68</v>
@@ -827,13 +827,13 @@
         <v>6</v>
       </c>
       <c r="B15">
-        <v>103.2692266182532</v>
+        <v>93.31047777482208</v>
       </c>
       <c r="C15">
-        <v>103.1519237721811</v>
+        <v>93.20491656666901</v>
       </c>
       <c r="D15">
-        <v>0.1173028460721497</v>
+        <v>0.1055612081530626</v>
       </c>
       <c r="E15" t="s">
         <v>69</v>
@@ -844,13 +844,13 @@
         <v>7</v>
       </c>
       <c r="B16">
-        <v>96.07728454684298</v>
+        <v>96.0873820711391</v>
       </c>
       <c r="C16">
-        <v>96.02938091308665</v>
+        <v>96.0395235455366</v>
       </c>
       <c r="D16">
-        <v>0.04790363375632012</v>
+        <v>0.04785852560250703</v>
       </c>
       <c r="E16" t="s">
         <v>63</v>
@@ -861,13 +861,13 @@
         <v>7</v>
       </c>
       <c r="B17">
-        <v>72.14998402688487</v>
+        <v>72.15720106325075</v>
       </c>
       <c r="C17">
-        <v>72.06261338053741</v>
+        <v>72.06982043446787</v>
       </c>
       <c r="D17">
-        <v>0.08737064634745195</v>
+        <v>0.08738062878288133</v>
       </c>
       <c r="E17" t="s">
         <v>64</v>
@@ -878,13 +878,13 @@
         <v>7</v>
       </c>
       <c r="B18">
-        <v>123.1821785985844</v>
+        <v>123.1947224060987</v>
       </c>
       <c r="C18">
-        <v>131.5539553868444</v>
+        <v>131.5684974482242</v>
       </c>
       <c r="D18">
-        <v>-8.371776788260007</v>
+        <v>-8.373775042125473</v>
       </c>
       <c r="E18" t="s">
         <v>65</v>
@@ -895,13 +895,13 @@
         <v>7</v>
       </c>
       <c r="B19">
-        <v>84.37449067229173</v>
+        <v>84.38312280669099</v>
       </c>
       <c r="C19">
-        <v>84.27009809399169</v>
+        <v>84.27871832441537</v>
       </c>
       <c r="D19">
-        <v>0.1043925783000361</v>
+        <v>0.1044044822756263</v>
       </c>
       <c r="E19" t="s">
         <v>66</v>
@@ -912,13 +912,13 @@
         <v>7</v>
       </c>
       <c r="B20">
-        <v>101.0636977829673</v>
+        <v>101.0739672670428</v>
       </c>
       <c r="C20">
-        <v>103.7382165570747</v>
+        <v>103.7493911069637</v>
       </c>
       <c r="D20">
-        <v>-2.674518774107383</v>
+        <v>-2.675423839920924</v>
       </c>
       <c r="E20" t="s">
         <v>67</v>
@@ -929,13 +929,13 @@
         <v>7</v>
       </c>
       <c r="B21">
-        <v>91.34365758573638</v>
+        <v>91.35313935204866</v>
       </c>
       <c r="C21">
-        <v>91.62430424202047</v>
+        <v>91.63397321133549</v>
       </c>
       <c r="D21">
-        <v>-0.280646656284091</v>
+        <v>-0.2808338592868296</v>
       </c>
       <c r="E21" t="s">
         <v>68</v>
@@ -946,13 +946,13 @@
         <v>7</v>
       </c>
       <c r="B22">
-        <v>100.7264989854941</v>
+        <v>100.7371193000324</v>
       </c>
       <c r="C22">
-        <v>100.6746144959441</v>
+        <v>100.6852561861928</v>
       </c>
       <c r="D22">
-        <v>0.05188448954997682</v>
+        <v>0.05186311383967279</v>
       </c>
       <c r="E22" t="s">
         <v>69</v>
@@ -963,13 +963,13 @@
         <v>8</v>
       </c>
       <c r="B23">
-        <v>96.22745766814171</v>
+        <v>96.23755522659482</v>
       </c>
       <c r="C23">
-        <v>96.18002297841115</v>
+        <v>96.19016607626369</v>
       </c>
       <c r="D23">
-        <v>0.04743468973056508</v>
+        <v>0.04738915033112789</v>
       </c>
       <c r="E23" t="s">
         <v>63</v>
@@ -980,13 +980,13 @@
         <v>8</v>
       </c>
       <c r="B24">
-        <v>72.31562050137848</v>
+        <v>72.32284012738599</v>
       </c>
       <c r="C24">
-        <v>72.22821850694849</v>
+        <v>72.23542814589148</v>
       </c>
       <c r="D24">
-        <v>0.08740199442998176</v>
+        <v>0.08741198149451179</v>
       </c>
       <c r="E24" t="s">
         <v>64</v>
@@ -997,13 +997,13 @@
         <v>8</v>
       </c>
       <c r="B25">
-        <v>123.2690407914781</v>
+        <v>123.2815701511858</v>
       </c>
       <c r="C25">
-        <v>131.6630243615105</v>
+        <v>131.6775611695413</v>
       </c>
       <c r="D25">
-        <v>-8.393983570032375</v>
+        <v>-8.395991018355446</v>
       </c>
       <c r="E25" t="s">
         <v>65</v>
@@ -1014,13 +1014,13 @@
         <v>8</v>
       </c>
       <c r="B26">
-        <v>84.53943683780454</v>
+        <v>84.54807156169649</v>
       </c>
       <c r="C26">
-        <v>84.43501342948099</v>
+        <v>84.44363624581592</v>
       </c>
       <c r="D26">
-        <v>0.1044234083235551</v>
+        <v>0.1044353158805649</v>
       </c>
       <c r="E26" t="s">
         <v>66</v>
@@ -1031,13 +1031,13 @@
         <v>8</v>
       </c>
       <c r="B27">
-        <v>101.1879053782059</v>
+        <v>101.1981675639944</v>
       </c>
       <c r="C27">
-        <v>103.8728901129752</v>
+        <v>103.8840628139921</v>
       </c>
       <c r="D27">
-        <v>-2.684984734769301</v>
+        <v>-2.685895249997685</v>
       </c>
       <c r="E27" t="s">
         <v>67</v>
@@ -1048,13 +1048,13 @@
         <v>8</v>
       </c>
       <c r="B28">
-        <v>91.49032300834574</v>
+        <v>91.49980348368406</v>
       </c>
       <c r="C28">
-        <v>91.7734681124123</v>
+        <v>91.78313723321827</v>
       </c>
       <c r="D28">
-        <v>-0.2831451040665627</v>
+        <v>-0.2833337495342079</v>
       </c>
       <c r="E28" t="s">
         <v>68</v>
@@ -1065,13 +1065,13 @@
         <v>8</v>
       </c>
       <c r="B29">
-        <v>100.8786178822768</v>
+        <v>100.8892387842838</v>
       </c>
       <c r="C29">
-        <v>100.8268728694112</v>
+        <v>100.8375153602018</v>
       </c>
       <c r="D29">
-        <v>0.05174501286559519</v>
+        <v>0.05172342408204145</v>
       </c>
       <c r="E29" t="s">
         <v>69</v>
@@ -1082,13 +1082,13 @@
         <v>9</v>
       </c>
       <c r="B30">
-        <v>96.30796145237021</v>
+        <v>96.31805870373194</v>
       </c>
       <c r="C30">
-        <v>96.26053788014993</v>
+        <v>96.27068090419684</v>
       </c>
       <c r="D30">
-        <v>0.04742357222028204</v>
+        <v>0.04737779953509857</v>
       </c>
       <c r="E30" t="s">
         <v>63</v>
@@ -1099,13 +1099,13 @@
         <v>9</v>
       </c>
       <c r="B31">
-        <v>72.40074071683797</v>
+        <v>72.40796092102532</v>
       </c>
       <c r="C31">
-        <v>72.31333164477174</v>
+        <v>72.32054186128596</v>
       </c>
       <c r="D31">
-        <v>0.0874090720662366</v>
+        <v>0.0874190597393607</v>
       </c>
       <c r="E31" t="s">
         <v>64</v>
@@ -1116,13 +1116,13 @@
         <v>9</v>
       </c>
       <c r="B32">
-        <v>123.318638888538</v>
+        <v>123.3311600615986</v>
       </c>
       <c r="C32">
-        <v>131.7315127552218</v>
+        <v>131.7460478365371</v>
       </c>
       <c r="D32">
-        <v>-8.412873866683796</v>
+        <v>-8.414887774938521</v>
       </c>
       <c r="E32" t="s">
         <v>65</v>
@@ -1133,13 +1133,13 @@
         <v>9</v>
       </c>
       <c r="B33">
-        <v>84.62384443387523</v>
+        <v>84.63247963118317</v>
       </c>
       <c r="C33">
-        <v>84.51941412064576</v>
+        <v>84.52803741034249</v>
       </c>
       <c r="D33">
-        <v>0.1044303132294715</v>
+        <v>0.1044422208406814</v>
       </c>
       <c r="E33" t="s">
         <v>66</v>
@@ -1150,13 +1150,13 @@
         <v>9</v>
       </c>
       <c r="B34">
-        <v>101.2580754335972</v>
+        <v>101.2683335930186</v>
       </c>
       <c r="C34">
-        <v>103.9491818941398</v>
+        <v>103.960353938079</v>
       </c>
       <c r="D34">
-        <v>-2.691106460542571</v>
+        <v>-2.692020345060413</v>
       </c>
       <c r="E34" t="s">
         <v>67</v>
@@ -1167,13 +1167,13 @@
         <v>9</v>
       </c>
       <c r="B35">
-        <v>91.57004233190094</v>
+        <v>91.57952192813079</v>
       </c>
       <c r="C35">
-        <v>91.85392925115049</v>
+        <v>91.86359828908215</v>
       </c>
       <c r="D35">
-        <v>-0.2838869192495537</v>
+        <v>-0.2840763609513601</v>
       </c>
       <c r="E35" t="s">
         <v>68</v>
@@ -1184,13 +1184,13 @@
         <v>9</v>
       </c>
       <c r="B36">
-        <v>100.9591920924578</v>
+        <v>100.9698128120773</v>
       </c>
       <c r="C36">
-        <v>100.9073952734782</v>
+        <v>100.9180376975664</v>
       </c>
       <c r="D36">
-        <v>0.05179681897965338</v>
+        <v>0.05177511451091732</v>
       </c>
       <c r="E36" t="s">
         <v>69</v>
@@ -1201,13 +1201,13 @@
         <v>10</v>
       </c>
       <c r="B37">
-        <v>99.55225107759921</v>
+        <v>88.37446227582153</v>
       </c>
       <c r="C37">
-        <v>99.45503188770415</v>
+        <v>88.28607311972657</v>
       </c>
       <c r="D37">
-        <v>0.09721918989505696</v>
+        <v>0.08838915609496212</v>
       </c>
       <c r="E37" t="s">
         <v>63</v>
@@ -1218,13 +1218,13 @@
         <v>10</v>
       </c>
       <c r="B38">
-        <v>98.28325736621581</v>
+        <v>79.01753819654715</v>
       </c>
       <c r="C38">
-        <v>98.19070471200973</v>
+        <v>78.93884863338364</v>
       </c>
       <c r="D38">
-        <v>0.09255265420607373</v>
+        <v>0.07868956316350761</v>
       </c>
       <c r="E38" t="s">
         <v>64</v>
@@ -1235,13 +1235,13 @@
         <v>10</v>
       </c>
       <c r="B39">
-        <v>101.3855180917988</v>
+        <v>98.89597929644924</v>
       </c>
       <c r="C39">
-        <v>101.2828965611392</v>
+        <v>98.79667304354521</v>
       </c>
       <c r="D39">
-        <v>0.1026215306596328</v>
+        <v>0.09930625290402872</v>
       </c>
       <c r="E39" t="s">
         <v>65</v>
@@ -1252,13 +1252,13 @@
         <v>10</v>
       </c>
       <c r="B40">
-        <v>98.3810376306275</v>
+        <v>89.15278566485262</v>
       </c>
       <c r="C40">
-        <v>98.28360319441096</v>
+        <v>89.06364916649731</v>
       </c>
       <c r="D40">
-        <v>0.09743443621654535</v>
+        <v>0.0891364983553018</v>
       </c>
       <c r="E40" t="s">
         <v>66</v>
@@ -1269,13 +1269,13 @@
         <v>10</v>
       </c>
       <c r="B41">
-        <v>100.5299300036076</v>
+        <v>85.6407876441604</v>
       </c>
       <c r="C41">
-        <v>100.4338182215674</v>
+        <v>85.55517390949241</v>
       </c>
       <c r="D41">
-        <v>0.09611178204018245</v>
+        <v>0.08561373466798727</v>
       </c>
       <c r="E41" t="s">
         <v>67</v>
@@ -1286,13 +1286,13 @@
         <v>10</v>
       </c>
       <c r="B42">
-        <v>100.0012479374046</v>
+        <v>82.42394512894987</v>
       </c>
       <c r="C42">
-        <v>99.90674897737416</v>
+        <v>82.34167050512636</v>
       </c>
       <c r="D42">
-        <v>0.09449896003040692</v>
+        <v>0.08227462382350836</v>
       </c>
       <c r="E42" t="s">
         <v>68</v>
@@ -1303,13 +1303,13 @@
         <v>10</v>
       </c>
       <c r="B43">
-        <v>99.27223824851229</v>
+        <v>94.76646612471112</v>
       </c>
       <c r="C43">
-        <v>99.172010019773</v>
+        <v>94.67150347292613</v>
       </c>
       <c r="D43">
-        <v>0.1002282287392973</v>
+        <v>0.0949626517849822</v>
       </c>
       <c r="E43" t="s">
         <v>69</v>
@@ -1320,13 +1320,13 @@
         <v>11</v>
       </c>
       <c r="B44">
-        <v>101.7249160236879</v>
+        <v>87.61504534942506</v>
       </c>
       <c r="C44">
-        <v>101.6191121329918</v>
+        <v>87.52139258207693</v>
       </c>
       <c r="D44">
-        <v>0.1058038906960803</v>
+        <v>0.09365276734813222</v>
       </c>
       <c r="E44" t="s">
         <v>63</v>
@@ -1337,13 +1337,13 @@
         <v>11</v>
       </c>
       <c r="B45">
-        <v>100.8195818586646</v>
+        <v>77.03818280215367</v>
       </c>
       <c r="C45">
-        <v>100.7187746127366</v>
+        <v>76.95635380539592</v>
       </c>
       <c r="D45">
-        <v>0.1008072459280385</v>
+        <v>0.08182899675774991</v>
       </c>
       <c r="E45" t="s">
         <v>64</v>
@@ -1354,13 +1354,13 @@
         <v>11</v>
       </c>
       <c r="B46">
-        <v>103.1547967289418</v>
+        <v>99.74069203692518</v>
       </c>
       <c r="C46">
-        <v>103.0432094733371</v>
+        <v>99.63346682974144</v>
       </c>
       <c r="D46">
-        <v>0.1115872556047321</v>
+        <v>0.1072252071837454</v>
       </c>
       <c r="E46" t="s">
         <v>65</v>
@@ -1371,13 +1371,13 @@
         <v>11</v>
       </c>
       <c r="B47">
-        <v>101.0222889814896</v>
+        <v>87.69574114649237</v>
       </c>
       <c r="C47">
-        <v>100.915696665837</v>
+        <v>87.60208901737445</v>
       </c>
       <c r="D47">
-        <v>0.1065923156526338</v>
+        <v>0.09365212911791332</v>
       </c>
       <c r="E47" t="s">
         <v>66</v>
@@ -1388,13 +1388,13 @@
         <v>11</v>
       </c>
       <c r="B48">
-        <v>102.4030674014402</v>
+        <v>85.2911519355945</v>
       </c>
       <c r="C48">
-        <v>102.2989080955252</v>
+        <v>85.20000823323899</v>
       </c>
       <c r="D48">
-        <v>0.1041593059150046</v>
+        <v>0.0911437023555095</v>
       </c>
       <c r="E48" t="s">
         <v>67</v>
@@ -1405,13 +1405,13 @@
         <v>11</v>
       </c>
       <c r="B49">
-        <v>102.0536096239265</v>
+        <v>81.56129064794052</v>
       </c>
       <c r="C49">
-        <v>101.9511166997827</v>
+        <v>81.47432385688894</v>
       </c>
       <c r="D49">
-        <v>0.1024929241437889</v>
+        <v>0.08696679105158012</v>
       </c>
       <c r="E49" t="s">
         <v>68</v>
@@ -1422,13 +1422,13 @@
         <v>11</v>
       </c>
       <c r="B50">
-        <v>101.6492849672439</v>
+        <v>94.13305533124489</v>
       </c>
       <c r="C50">
-        <v>101.5397508216573</v>
+        <v>94.03219659762779</v>
       </c>
       <c r="D50">
-        <v>0.1095341455866077</v>
+        <v>0.1008587336171018</v>
       </c>
       <c r="E50" t="s">
         <v>69</v>
@@ -1439,13 +1439,13 @@
         <v>12</v>
       </c>
       <c r="B51">
-        <v>98.84770517359279</v>
+        <v>98.85693377104015</v>
       </c>
       <c r="C51">
-        <v>98.8922126558614</v>
+        <v>98.90208347664061</v>
       </c>
       <c r="D51">
-        <v>-0.04450748226861378</v>
+        <v>-0.0451497056004655</v>
       </c>
       <c r="E51" t="s">
         <v>63</v>
@@ -1456,13 +1456,13 @@
         <v>12</v>
       </c>
       <c r="B52">
-        <v>82.43401067209508</v>
+        <v>82.44210559726139</v>
       </c>
       <c r="C52">
-        <v>82.33599331174439</v>
+        <v>82.34407796277968</v>
       </c>
       <c r="D52">
-        <v>0.09801736035069553</v>
+        <v>0.09802763448170992</v>
       </c>
       <c r="E52" t="s">
         <v>64</v>
@@ -1473,13 +1473,13 @@
         <v>12</v>
       </c>
       <c r="B53">
-        <v>105.1098463445913</v>
+        <v>105.1128245192902</v>
       </c>
       <c r="C53">
-        <v>119.2858125851054</v>
+        <v>119.2978931893979</v>
       </c>
       <c r="D53">
-        <v>-14.17596624051416</v>
+        <v>-14.18506867010773</v>
       </c>
       <c r="E53" t="s">
         <v>65</v>
@@ -1490,13 +1490,13 @@
         <v>12</v>
       </c>
       <c r="B54">
-        <v>95.43068968099956</v>
+        <v>95.44010060775334</v>
       </c>
       <c r="C54">
-        <v>95.32671592848472</v>
+        <v>95.33616857135027</v>
       </c>
       <c r="D54">
-        <v>0.1039737525148468</v>
+        <v>0.1039320364030658</v>
       </c>
       <c r="E54" t="s">
         <v>66</v>
@@ -1507,13 +1507,13 @@
         <v>12</v>
       </c>
       <c r="B55">
-        <v>98.18780037899438</v>
+        <v>98.19477500788254</v>
       </c>
       <c r="C55">
-        <v>98.93130730334087</v>
+        <v>98.94121528148678</v>
       </c>
       <c r="D55">
-        <v>-0.7435069243464909</v>
+        <v>-0.7464402736042359</v>
       </c>
       <c r="E55" t="s">
         <v>67</v>
@@ -1524,13 +1524,13 @@
         <v>12</v>
       </c>
       <c r="B56">
-        <v>92.57844728681931</v>
+        <v>92.5874634322206</v>
       </c>
       <c r="C56">
-        <v>92.49633756560749</v>
+        <v>92.50554732150455</v>
       </c>
       <c r="D56">
-        <v>0.08210972121182181</v>
+        <v>0.08191611071605109</v>
       </c>
       <c r="E56" t="s">
         <v>68</v>
@@ -1541,13 +1541,13 @@
         <v>12</v>
       </c>
       <c r="B57">
-        <v>104.1692127275694</v>
+        <v>104.1750033034132</v>
       </c>
       <c r="C57">
-        <v>105.7434428628753</v>
+        <v>105.7540226638049</v>
       </c>
       <c r="D57">
-        <v>-1.574230135305967</v>
+        <v>-1.579019360391698</v>
       </c>
       <c r="E57" t="s">
         <v>69</v>
@@ -1558,13 +1558,13 @@
         <v>13</v>
       </c>
       <c r="B58">
-        <v>99.57897761498015</v>
+        <v>99.58824786548189</v>
       </c>
       <c r="C58">
-        <v>99.61781340288334</v>
+        <v>99.62765858831003</v>
       </c>
       <c r="D58">
-        <v>-0.03883578790319575</v>
+        <v>-0.03941072282813707</v>
       </c>
       <c r="E58" t="s">
         <v>63</v>
@@ -1575,13 +1575,13 @@
         <v>13</v>
       </c>
       <c r="B59">
-        <v>83.3613303912599</v>
+        <v>83.3694309271886</v>
       </c>
       <c r="C59">
-        <v>83.26324473824684</v>
+        <v>83.27133504588286</v>
       </c>
       <c r="D59">
-        <v>0.09808565301305805</v>
+        <v>0.09809588130573843</v>
       </c>
       <c r="E59" t="s">
         <v>64</v>
@@ -1592,13 +1592,13 @@
         <v>13</v>
       </c>
       <c r="B60">
-        <v>105.2427825792741</v>
+        <v>105.2454230198436</v>
       </c>
       <c r="C60">
-        <v>119.6902148336369</v>
+        <v>119.7022230878312</v>
       </c>
       <c r="D60">
-        <v>-14.44743225436278</v>
+        <v>-14.45680006798756</v>
       </c>
       <c r="E60" t="s">
         <v>65</v>
@@ -1609,13 +1609,13 @@
         <v>13</v>
       </c>
       <c r="B61">
-        <v>96.33594645675997</v>
+        <v>96.34536974466447</v>
       </c>
       <c r="C61">
-        <v>96.23145185006493</v>
+        <v>96.24090065435361</v>
       </c>
       <c r="D61">
-        <v>0.1044946066950416</v>
+        <v>0.1044690903108574</v>
       </c>
       <c r="E61" t="s">
         <v>66</v>
@@ -1626,13 +1626,13 @@
         <v>13</v>
       </c>
       <c r="B62">
-        <v>98.86710790709704</v>
+        <v>98.8739916535918</v>
       </c>
       <c r="C62">
-        <v>99.51618868204066</v>
+        <v>99.52605539793429</v>
       </c>
       <c r="D62">
-        <v>-0.6490807749436271</v>
+        <v>-0.6520637443424846</v>
       </c>
       <c r="E62" t="s">
         <v>67</v>
@@ -1643,13 +1643,13 @@
         <v>13</v>
       </c>
       <c r="B63">
-        <v>93.27803342218539</v>
+        <v>93.28706407228421</v>
       </c>
       <c r="C63">
-        <v>93.18727311147114</v>
+        <v>93.19645687702705</v>
       </c>
       <c r="D63">
-        <v>0.09076031071424495</v>
+        <v>0.09060719525716365</v>
       </c>
       <c r="E63" t="s">
         <v>68</v>
@@ -1660,13 +1660,13 @@
         <v>13</v>
       </c>
       <c r="B64">
-        <v>104.6150179360975</v>
+        <v>104.6205569960759</v>
       </c>
       <c r="C64">
-        <v>106.5076012280771</v>
+        <v>106.5181559736313</v>
       </c>
       <c r="D64">
-        <v>-1.892583291979562</v>
+        <v>-1.897598977555376</v>
       </c>
       <c r="E64" t="s">
         <v>69</v>
@@ -1677,13 +1677,13 @@
         <v>14</v>
       </c>
       <c r="B65">
-        <v>99.62385383477128</v>
+        <v>99.63313074564924</v>
       </c>
       <c r="C65">
-        <v>99.6609749003029</v>
+        <v>99.67081786330752</v>
       </c>
       <c r="D65">
-        <v>-0.03712106553162187</v>
+        <v>-0.03768711765827959</v>
       </c>
       <c r="E65" t="s">
         <v>63</v>
@@ -1694,13 +1694,13 @@
         <v>14</v>
       </c>
       <c r="B66">
-        <v>83.41687970535173</v>
+        <v>83.42497986085765</v>
       </c>
       <c r="C66">
-        <v>83.31879863968439</v>
+        <v>83.32688857018495</v>
       </c>
       <c r="D66">
-        <v>0.09808106566734409</v>
+        <v>0.09809129067269851</v>
       </c>
       <c r="E66" t="s">
         <v>64</v>
@@ -1711,13 +1711,13 @@
         <v>14</v>
       </c>
       <c r="B67">
-        <v>105.2235468659093</v>
+        <v>105.2261459876978</v>
       </c>
       <c r="C67">
-        <v>119.7141584884807</v>
+        <v>119.7261618004958</v>
       </c>
       <c r="D67">
-        <v>-14.49061162257139</v>
+        <v>-14.50001581279803</v>
       </c>
       <c r="E67" t="s">
         <v>65</v>
@@ -1728,13 +1728,13 @@
         <v>14</v>
       </c>
       <c r="B68">
-        <v>96.38935702666858</v>
+        <v>96.39878114013763</v>
       </c>
       <c r="C68">
-        <v>96.28459589770934</v>
+        <v>96.29404369846223</v>
       </c>
       <c r="D68">
-        <v>0.1047611289592396</v>
+        <v>0.1047374416753968</v>
       </c>
       <c r="E68" t="s">
         <v>66</v>
@@ -1745,13 +1745,13 @@
         <v>14</v>
       </c>
       <c r="B69">
-        <v>98.91399788419535</v>
+        <v>98.92087215249826</v>
       </c>
       <c r="C69">
-        <v>99.55174750945126</v>
+        <v>99.56161114980507</v>
       </c>
       <c r="D69">
-        <v>-0.6377496252559069</v>
+        <v>-0.6407389973068121</v>
       </c>
       <c r="E69" t="s">
         <v>67</v>
@@ -1762,13 +1762,13 @@
         <v>14</v>
       </c>
       <c r="B70">
-        <v>93.3209279131063</v>
+        <v>93.32996133861703</v>
       </c>
       <c r="C70">
-        <v>93.22912671690634</v>
+        <v>93.23830829230479</v>
       </c>
       <c r="D70">
-        <v>0.09180119619996674</v>
+        <v>0.09165304631223137</v>
       </c>
       <c r="E70" t="s">
         <v>68</v>
@@ -1779,13 +1779,13 @@
         <v>14</v>
       </c>
       <c r="B71">
-        <v>104.6276718480467</v>
+        <v>104.6331796025454</v>
       </c>
       <c r="C71">
-        <v>106.552247441821</v>
+        <v>106.5627999419577</v>
       </c>
       <c r="D71">
-        <v>-1.924575593774321</v>
+        <v>-1.929620339412224</v>
       </c>
       <c r="E71" t="s">
         <v>69</v>
@@ -1796,13 +1796,13 @@
         <v>15</v>
       </c>
       <c r="B72">
-        <v>96.01772077750338</v>
+        <v>72.50690857839989</v>
       </c>
       <c r="C72">
-        <v>95.92796072599644</v>
+        <v>72.41361652806917</v>
       </c>
       <c r="D72">
-        <v>0.08976005150694277</v>
+        <v>0.0932920503307173</v>
       </c>
       <c r="E72" t="s">
         <v>63</v>
@@ -1813,13 +1813,13 @@
         <v>15</v>
       </c>
       <c r="B73">
-        <v>94.73751953279063</v>
+        <v>58.03336271275611</v>
       </c>
       <c r="C73">
-        <v>94.63991586196512</v>
+        <v>57.96018511178455</v>
       </c>
       <c r="D73">
-        <v>0.09760367082550658</v>
+        <v>0.07317760097156167</v>
       </c>
       <c r="E73" t="s">
         <v>64</v>
@@ -1830,13 +1830,13 @@
         <v>15</v>
       </c>
       <c r="B74">
-        <v>98.17707257970754</v>
+        <v>91.04101077344455</v>
       </c>
       <c r="C74">
-        <v>98.86558860137328</v>
+        <v>90.92876116645532</v>
       </c>
       <c r="D74">
-        <v>-0.688516021665734</v>
+        <v>0.1122496069892378</v>
       </c>
       <c r="E74" t="s">
         <v>65</v>
@@ -1847,13 +1847,13 @@
         <v>15</v>
       </c>
       <c r="B75">
-        <v>91.92046861581468</v>
+        <v>67.94005089009451</v>
       </c>
       <c r="C75">
-        <v>91.83023484362694</v>
+        <v>67.85325367027372</v>
       </c>
       <c r="D75">
-        <v>0.09023377218774442</v>
+        <v>0.08679721982079514</v>
       </c>
       <c r="E75" t="s">
         <v>66</v>
@@ -1864,13 +1864,13 @@
         <v>15</v>
       </c>
       <c r="B76">
-        <v>100.0479421354363</v>
+        <v>74.03763430324058</v>
       </c>
       <c r="C76">
-        <v>100.2101138709991</v>
+        <v>73.94206790641491</v>
       </c>
       <c r="D76">
-        <v>-0.1621717355627226</v>
+        <v>0.09556639682567436</v>
       </c>
       <c r="E76" t="s">
         <v>67</v>
@@ -1881,13 +1881,13 @@
         <v>15</v>
       </c>
       <c r="B77">
-        <v>99.21149427980595</v>
+        <v>68.12929791451522</v>
       </c>
       <c r="C77">
-        <v>99.22003042665956</v>
+        <v>68.04196017714062</v>
       </c>
       <c r="D77">
-        <v>-0.008536146853614923</v>
+        <v>0.08733773737459671</v>
       </c>
       <c r="E77" t="s">
         <v>68</v>
@@ -1898,13 +1898,13 @@
         <v>15</v>
       </c>
       <c r="B78">
-        <v>92.93434258622409</v>
+        <v>77.18175437109248</v>
       </c>
       <c r="C78">
-        <v>92.90653684424497</v>
+        <v>77.0820975852088</v>
       </c>
       <c r="D78">
-        <v>0.02780574197912244</v>
+        <v>0.09965678588368121</v>
       </c>
       <c r="E78" t="s">
         <v>69</v>
@@ -1915,13 +1915,13 @@
         <v>16</v>
       </c>
       <c r="B79">
-        <v>103.9404112261997</v>
+        <v>86.52724841860909</v>
       </c>
       <c r="C79">
-        <v>103.8273463373159</v>
+        <v>86.42904522660545</v>
       </c>
       <c r="D79">
-        <v>0.1130648888837413</v>
+        <v>0.0982031920036377</v>
       </c>
       <c r="E79" t="s">
         <v>63</v>
@@ -1932,13 +1932,13 @@
         <v>16</v>
       </c>
       <c r="B80">
-        <v>103.3465577913727</v>
+        <v>74.52274330135653</v>
       </c>
       <c r="C80">
-        <v>103.2403026764264</v>
+        <v>74.4390000592737</v>
       </c>
       <c r="D80">
-        <v>0.1062551149463218</v>
+        <v>0.08374324208283213</v>
       </c>
       <c r="E80" t="s">
         <v>64</v>
@@ -1949,13 +1949,13 @@
         <v>16</v>
       </c>
       <c r="B81">
-        <v>105.3783713518261</v>
+        <v>100.6335600020557</v>
       </c>
       <c r="C81">
-        <v>105.2572502688447</v>
+        <v>100.5183447762463</v>
       </c>
       <c r="D81">
-        <v>0.1211210829814036</v>
+        <v>0.1152152258094219</v>
       </c>
       <c r="E81" t="s">
         <v>65</v>
@@ -1966,13 +1966,13 @@
         <v>16</v>
       </c>
       <c r="B82">
-        <v>102.37458698058</v>
+        <v>85.47598766225333</v>
       </c>
       <c r="C82">
-        <v>102.2610170570968</v>
+        <v>85.37914416970932</v>
       </c>
       <c r="D82">
-        <v>0.1135699234832401</v>
+        <v>0.0968434925440107</v>
       </c>
       <c r="E82" t="s">
         <v>66</v>
@@ -1983,13 +1983,13 @@
         <v>16</v>
       </c>
       <c r="B83">
-        <v>105.5962973710966</v>
+        <v>85.00137954412477</v>
       </c>
       <c r="C83">
-        <v>105.4849297440026</v>
+        <v>84.90492278015843</v>
       </c>
       <c r="D83">
-        <v>0.1113676270939834</v>
+        <v>0.09645676396634428</v>
       </c>
       <c r="E83" t="s">
         <v>67</v>
@@ -2000,13 +2000,13 @@
         <v>16</v>
       </c>
       <c r="B84">
-        <v>105.2816319264011</v>
+        <v>80.6181396484771</v>
       </c>
       <c r="C84">
-        <v>105.1726077931943</v>
+        <v>80.52697109104169</v>
       </c>
       <c r="D84">
-        <v>0.1090241332068445</v>
+        <v>0.09116855743540953</v>
       </c>
       <c r="E84" t="s">
         <v>68</v>
@@ -2017,13 +2017,13 @@
         <v>16</v>
       </c>
       <c r="B85">
-        <v>102.9754299581952</v>
+        <v>92.89137999020053</v>
       </c>
       <c r="C85">
-        <v>102.8577702911113</v>
+        <v>92.78559395993679</v>
       </c>
       <c r="D85">
-        <v>0.1176596670838705</v>
+        <v>0.1057860302637437</v>
       </c>
       <c r="E85" t="s">
         <v>69</v>
@@ -2034,13 +2034,13 @@
         <v>17</v>
       </c>
       <c r="B86">
-        <v>104.8984881404407</v>
+        <v>104.9060519405605</v>
       </c>
       <c r="C86">
-        <v>106.7044007164347</v>
+        <v>106.7151637579515</v>
       </c>
       <c r="D86">
-        <v>-1.805912575993943</v>
+        <v>-1.809111817391042</v>
       </c>
       <c r="E86" t="s">
         <v>63</v>
@@ -2051,13 +2051,13 @@
         <v>17</v>
       </c>
       <c r="B87">
-        <v>87.39869666119598</v>
+        <v>87.40730075026894</v>
       </c>
       <c r="C87">
-        <v>87.29497263358331</v>
+        <v>87.30356668987594</v>
       </c>
       <c r="D87">
-        <v>0.103724027612671</v>
+        <v>0.103734060393009</v>
       </c>
       <c r="E87" t="s">
         <v>64</v>
@@ -2068,13 +2068,13 @@
         <v>17</v>
       </c>
       <c r="B88">
-        <v>111.7146170687134</v>
+        <v>111.7205180043511</v>
       </c>
       <c r="C88">
-        <v>131.3844327380201</v>
+        <v>131.3979710671924</v>
       </c>
       <c r="D88">
-        <v>-19.66981566930679</v>
+        <v>-19.67745306284131</v>
       </c>
       <c r="E88" t="s">
         <v>65</v>
@@ -2085,13 +2085,13 @@
         <v>17</v>
       </c>
       <c r="B89">
-        <v>101.2828205326606</v>
+        <v>101.2925319955577</v>
       </c>
       <c r="C89">
-        <v>101.2827346053352</v>
+        <v>101.2928398897354</v>
       </c>
       <c r="D89">
-        <v>8.592732537238135E-05</v>
+        <v>-0.0003078941776522015</v>
       </c>
       <c r="E89" t="s">
         <v>66</v>
@@ -2102,13 +2102,13 @@
         <v>17</v>
       </c>
       <c r="B90">
-        <v>102.347260527848</v>
+        <v>102.3533590157611</v>
       </c>
       <c r="C90">
-        <v>108.0848724085326</v>
+        <v>108.0958413912315</v>
       </c>
       <c r="D90">
-        <v>-5.737611880684611</v>
+        <v>-5.742482375470317</v>
       </c>
       <c r="E90" t="s">
         <v>67</v>
@@ -2119,13 +2119,13 @@
         <v>17</v>
       </c>
       <c r="B91">
-        <v>98.84820250192381</v>
+        <v>98.85607177674574</v>
       </c>
       <c r="C91">
-        <v>100.2368949387817</v>
+        <v>100.2469798380881</v>
       </c>
       <c r="D91">
-        <v>-1.388692436857852</v>
+        <v>-1.390908061342316</v>
       </c>
       <c r="E91" t="s">
         <v>68</v>
@@ -2136,13 +2136,13 @@
         <v>17</v>
       </c>
       <c r="B92">
-        <v>110.4213057157285</v>
+        <v>110.4284727252258</v>
       </c>
       <c r="C92">
-        <v>113.6048992418702</v>
+        <v>113.6163865913574</v>
       </c>
       <c r="D92">
-        <v>-3.183593526141735</v>
+        <v>-3.187913866131609</v>
       </c>
       <c r="E92" t="s">
         <v>69</v>
@@ -2153,13 +2153,13 @@
         <v>18</v>
       </c>
       <c r="B93">
-        <v>105.1862757371466</v>
+        <v>105.1937845505193</v>
       </c>
       <c r="C93">
-        <v>107.0262792301261</v>
+        <v>107.0370347979289</v>
       </c>
       <c r="D93">
-        <v>-1.840003492979562</v>
+        <v>-1.843250247409628</v>
       </c>
       <c r="E93" t="s">
         <v>63</v>
@@ -2170,13 +2170,13 @@
         <v>18</v>
       </c>
       <c r="B94">
-        <v>87.79714421570989</v>
+        <v>87.80575262223469</v>
       </c>
       <c r="C94">
-        <v>87.69334799494605</v>
+        <v>87.70194630143386</v>
       </c>
       <c r="D94">
-        <v>0.1037962207638401</v>
+        <v>0.1038063208008282</v>
       </c>
       <c r="E94" t="s">
         <v>64</v>
@@ -2187,13 +2187,13 @@
         <v>18</v>
       </c>
       <c r="B95">
-        <v>111.8376381404162</v>
+        <v>111.8434402356179</v>
       </c>
       <c r="C95">
-        <v>131.5752410014853</v>
+        <v>131.5887529707466</v>
       </c>
       <c r="D95">
-        <v>-19.73760286106911</v>
+        <v>-19.74531273512872</v>
       </c>
       <c r="E95" t="s">
         <v>65</v>
@@ -2204,13 +2204,13 @@
         <v>18</v>
       </c>
       <c r="B96">
-        <v>101.6720037015705</v>
+        <v>101.6817180019322</v>
       </c>
       <c r="C96">
-        <v>101.6823396090849</v>
+        <v>101.6924472356592</v>
       </c>
       <c r="D96">
-        <v>-0.01033590751440272</v>
+        <v>-0.01072923372707635</v>
       </c>
       <c r="E96" t="s">
         <v>66</v>
@@ -2221,13 +2221,13 @@
         <v>18</v>
       </c>
       <c r="B97">
-        <v>102.632745940937</v>
+        <v>102.6387658809387</v>
       </c>
       <c r="C97">
-        <v>108.3396892335838</v>
+        <v>108.3506427544998</v>
       </c>
       <c r="D97">
-        <v>-5.706943292646741</v>
+        <v>-5.71187687356101</v>
       </c>
       <c r="E97" t="s">
         <v>67</v>
@@ -2238,13 +2238,13 @@
         <v>18</v>
       </c>
       <c r="B98">
-        <v>99.16582411787645</v>
+        <v>99.17365945398458</v>
       </c>
       <c r="C98">
-        <v>100.5363359182203</v>
+        <v>100.5464117099415</v>
       </c>
       <c r="D98">
-        <v>-1.370511800343877</v>
+        <v>-1.372752255956897</v>
       </c>
       <c r="E98" t="s">
         <v>68</v>
@@ -2255,13 +2255,13 @@
         <v>18</v>
       </c>
       <c r="B99">
-        <v>110.6475556783861</v>
+        <v>110.6546454799219</v>
       </c>
       <c r="C99">
-        <v>113.9519542543775</v>
+        <v>113.9634360361408</v>
       </c>
       <c r="D99">
-        <v>-3.304398575991456</v>
+        <v>-3.308790556218938</v>
       </c>
       <c r="E99" t="s">
         <v>69</v>
@@ -2272,13 +2272,13 @@
         <v>19</v>
       </c>
       <c r="B100">
-        <v>95.48660298126229</v>
+        <v>75.36246684023007</v>
       </c>
       <c r="C100">
-        <v>95.44327306106776</v>
+        <v>75.26738390657738</v>
       </c>
       <c r="D100">
-        <v>0.04332992019453741</v>
+        <v>0.09508293365269083</v>
       </c>
       <c r="E100" t="s">
         <v>63</v>
@@ -2289,13 +2289,13 @@
         <v>19</v>
       </c>
       <c r="B101">
-        <v>93.7319259057287</v>
+        <v>61.74925750099757</v>
       </c>
       <c r="C101">
-        <v>93.65790100485989</v>
+        <v>61.67237646482638</v>
       </c>
       <c r="D101">
-        <v>0.07402490086880675</v>
+        <v>0.07688103617119424</v>
       </c>
       <c r="E101" t="s">
         <v>64</v>
@@ -2306,13 +2306,13 @@
         <v>19</v>
       </c>
       <c r="B102">
-        <v>97.58561134658328</v>
+        <v>92.26619357357418</v>
       </c>
       <c r="C102">
-        <v>98.49546619648869</v>
+        <v>92.14959007695178</v>
       </c>
       <c r="D102">
-        <v>-0.9098548499054147</v>
+        <v>0.1166034966224032</v>
       </c>
       <c r="E102" t="s">
         <v>65</v>
@@ -2323,13 +2323,13 @@
         <v>19</v>
       </c>
       <c r="B103">
-        <v>92.9869463694335</v>
+        <v>71.98898681556766</v>
       </c>
       <c r="C103">
-        <v>92.94471898690271</v>
+        <v>71.89857142871456</v>
       </c>
       <c r="D103">
-        <v>0.04222738253078262</v>
+        <v>0.09041538685309547</v>
       </c>
       <c r="E103" t="s">
         <v>66</v>
@@ -2340,13 +2340,13 @@
         <v>19</v>
       </c>
       <c r="B104">
-        <v>97.56240250414623</v>
+        <v>75.82828646862804</v>
       </c>
       <c r="C104">
-        <v>97.87822083842035</v>
+        <v>75.73242640347435</v>
       </c>
       <c r="D104">
-        <v>-0.3158183342741125</v>
+        <v>0.09586006515368695</v>
       </c>
       <c r="E104" t="s">
         <v>67</v>
@@ -2357,13 +2357,13 @@
         <v>19</v>
       </c>
       <c r="B105">
-        <v>96.83658083106562</v>
+        <v>70.4802307198062</v>
       </c>
       <c r="C105">
-        <v>96.95341789566866</v>
+        <v>70.39153828796204</v>
       </c>
       <c r="D105">
-        <v>-0.1168370646030468</v>
+        <v>0.08869243184416575</v>
       </c>
       <c r="E105" t="s">
         <v>68</v>
@@ -2374,13 +2374,13 @@
         <v>19</v>
       </c>
       <c r="B106">
-        <v>94.13578040824737</v>
+        <v>80.59464889908031</v>
       </c>
       <c r="C106">
-        <v>94.21001462456701</v>
+        <v>80.49271022341516</v>
       </c>
       <c r="D106">
-        <v>-0.07423421631963834</v>
+        <v>0.1019386756651528</v>
       </c>
       <c r="E106" t="s">
         <v>69</v>
@@ -2391,13 +2391,13 @@
         <v>20</v>
       </c>
       <c r="B107">
-        <v>102.2548764078642</v>
+        <v>91.056720256291</v>
       </c>
       <c r="C107">
-        <v>102.1639332948339</v>
+        <v>90.97449995735786</v>
       </c>
       <c r="D107">
-        <v>0.09094311303029201</v>
+        <v>0.08222029893313731</v>
       </c>
       <c r="E107" t="s">
         <v>63</v>
@@ -2408,13 +2408,13 @@
         <v>20</v>
       </c>
       <c r="B108">
-        <v>102.368886410102</v>
+        <v>83.06603804171542</v>
       </c>
       <c r="C108">
-        <v>102.2804562303099</v>
+        <v>82.99124706397902</v>
       </c>
       <c r="D108">
-        <v>0.08843017979202727</v>
+        <v>0.07479097773639864</v>
       </c>
       <c r="E108" t="s">
         <v>64</v>
@@ -2425,13 +2425,13 @@
         <v>20</v>
       </c>
       <c r="B109">
-        <v>102.3671651629121</v>
+        <v>99.84671822037885</v>
       </c>
       <c r="C109">
-        <v>102.2734179852597</v>
+        <v>99.75631977431951</v>
       </c>
       <c r="D109">
-        <v>0.09374717765238927</v>
+        <v>0.09039844605933922</v>
       </c>
       <c r="E109" t="s">
         <v>65</v>
@@ -2442,13 +2442,13 @@
         <v>20</v>
       </c>
       <c r="B110">
-        <v>101.7096958603295</v>
+        <v>92.55703404105563</v>
       </c>
       <c r="C110">
-        <v>101.6179580612776</v>
+        <v>92.4734550782</v>
       </c>
       <c r="D110">
-        <v>0.09173779905188439</v>
+        <v>0.0835789628556256</v>
       </c>
       <c r="E110" t="s">
         <v>66</v>
@@ -2459,13 +2459,13 @@
         <v>20</v>
       </c>
       <c r="B111">
-        <v>102.9181338601868</v>
+        <v>87.91269018384962</v>
       </c>
       <c r="C111">
-        <v>102.8284075152933</v>
+        <v>87.8333572991849</v>
       </c>
       <c r="D111">
-        <v>0.08972634489353482</v>
+        <v>0.07933288466472277</v>
       </c>
       <c r="E111" t="s">
         <v>67</v>
@@ -2476,13 +2476,13 @@
         <v>20</v>
       </c>
       <c r="B112">
-        <v>102.9246113408304</v>
+        <v>85.23315400600768</v>
       </c>
       <c r="C112">
-        <v>102.8356973338008</v>
+        <v>85.15631507305359</v>
       </c>
       <c r="D112">
-        <v>0.08891400702960084</v>
+        <v>0.0768389329540895</v>
       </c>
       <c r="E112" t="s">
         <v>68</v>
@@ -2493,13 +2493,13 @@
         <v>20</v>
       </c>
       <c r="B113">
-        <v>101.7277533677134</v>
+        <v>97.28785249768831</v>
       </c>
       <c r="C113">
-        <v>101.6345672427153</v>
+        <v>97.19987051384116</v>
       </c>
       <c r="D113">
-        <v>0.09318612499812673</v>
+        <v>0.0879819838471434</v>
       </c>
       <c r="E113" t="s">
         <v>69</v>
@@ -2510,13 +2510,13 @@
         <v>21</v>
       </c>
       <c r="B114">
-        <v>95.64820239929452</v>
+        <v>75.50930035213678</v>
       </c>
       <c r="C114">
-        <v>95.60052139139654</v>
+        <v>75.41423508089437</v>
       </c>
       <c r="D114">
-        <v>0.04768100789797813</v>
+        <v>0.09506527124240449</v>
       </c>
       <c r="E114" t="s">
         <v>63</v>
@@ -2527,13 +2527,13 @@
         <v>21</v>
       </c>
       <c r="B115">
-        <v>93.96550537136601</v>
+        <v>61.93424235335238</v>
       </c>
       <c r="C115">
-        <v>93.89025651406405</v>
+        <v>61.85730390218247</v>
       </c>
       <c r="D115">
-        <v>0.07524885730195763</v>
+        <v>0.07693845116990872</v>
       </c>
       <c r="E115" t="s">
         <v>64</v>
@@ -2544,13 +2544,13 @@
         <v>21</v>
       </c>
       <c r="B116">
-        <v>97.67407262773919</v>
+        <v>92.3487582916725</v>
       </c>
       <c r="C116">
-        <v>98.57033096763369</v>
+        <v>92.23211076684602</v>
       </c>
       <c r="D116">
-        <v>-0.8962583398945014</v>
+        <v>0.116647524826476</v>
       </c>
       <c r="E116" t="s">
         <v>65</v>
@@ -2561,13 +2561,13 @@
         <v>21</v>
       </c>
       <c r="B117">
-        <v>93.1544987962383</v>
+        <v>72.17379592564417</v>
       </c>
       <c r="C117">
-        <v>93.10992093322707</v>
+        <v>72.08333887085365</v>
       </c>
       <c r="D117">
-        <v>0.04457786301122724</v>
+        <v>0.09045705479051946</v>
       </c>
       <c r="E117" t="s">
         <v>66</v>
@@ -2578,13 +2578,13 @@
         <v>21</v>
       </c>
       <c r="B118">
-        <v>97.74233553079529</v>
+        <v>75.94409481257482</v>
       </c>
       <c r="C118">
-        <v>98.04059636573558</v>
+        <v>75.8482972416972</v>
       </c>
       <c r="D118">
-        <v>-0.2982608349402938</v>
+        <v>0.09579757087762175</v>
       </c>
       <c r="E118" t="s">
         <v>67</v>
@@ -2595,13 +2595,13 @@
         <v>21</v>
       </c>
       <c r="B119">
-        <v>97.04268771214892</v>
+        <v>70.6174448253991</v>
       </c>
       <c r="C119">
-        <v>97.14675552170492</v>
+        <v>70.52877645990169</v>
       </c>
       <c r="D119">
-        <v>-0.1040678095559997</v>
+        <v>0.08866836549741208</v>
       </c>
       <c r="E119" t="s">
         <v>68</v>
@@ -2612,13 +2612,13 @@
         <v>21</v>
       </c>
       <c r="B120">
-        <v>94.26565255392909</v>
+        <v>80.75226418172353</v>
       </c>
       <c r="C120">
-        <v>94.33663570943423</v>
+        <v>80.65033566461204</v>
       </c>
       <c r="D120">
-        <v>-0.07098315550514656</v>
+        <v>0.1019285171114888</v>
       </c>
       <c r="E120" t="s">
         <v>69</v>
@@ -2629,13 +2629,13 @@
         <v>22</v>
       </c>
       <c r="B121">
-        <v>102.5014492513059</v>
+        <v>91.29798187112559</v>
       </c>
       <c r="C121">
-        <v>102.4111892937343</v>
+        <v>91.21635293996619</v>
       </c>
       <c r="D121">
-        <v>0.09025995757161809</v>
+        <v>0.08162893115940051</v>
       </c>
       <c r="E121" t="s">
         <v>63</v>
@@ -2646,13 +2646,13 @@
         <v>22</v>
       </c>
       <c r="B122">
-        <v>102.7495067579277</v>
+        <v>83.42058544404867</v>
       </c>
       <c r="C122">
-        <v>102.6616780733299</v>
+        <v>83.34621642007366</v>
       </c>
       <c r="D122">
-        <v>0.08782868459783799</v>
+        <v>0.07436902397500944</v>
       </c>
       <c r="E122" t="s">
         <v>64</v>
@@ -2663,13 +2663,13 @@
         <v>22</v>
       </c>
       <c r="B123">
-        <v>102.4753341745071</v>
+        <v>99.94963949250752</v>
       </c>
       <c r="C123">
-        <v>102.3823636579091</v>
+        <v>99.86003168931548</v>
       </c>
       <c r="D123">
-        <v>0.09297051659795841</v>
+        <v>0.0896078031920382</v>
       </c>
       <c r="E123" t="s">
         <v>65</v>
@@ -2680,13 +2680,13 @@
         <v>22</v>
       </c>
       <c r="B124">
-        <v>101.9242265925669</v>
+        <v>92.84592684474728</v>
       </c>
       <c r="C124">
-        <v>101.8331645411286</v>
+        <v>92.76290617631039</v>
       </c>
       <c r="D124">
-        <v>0.09106205143828561</v>
+        <v>0.08302066843688749</v>
       </c>
       <c r="E124" t="s">
         <v>66</v>
@@ -2697,13 +2697,13 @@
         <v>22</v>
       </c>
       <c r="B125">
-        <v>103.2227426124319</v>
+        <v>88.13076165466164</v>
       </c>
       <c r="C125">
-        <v>103.1336930512006</v>
+        <v>88.0520172545196</v>
       </c>
       <c r="D125">
-        <v>0.08904956123133445</v>
+        <v>0.07874440014204254</v>
       </c>
       <c r="E125" t="s">
         <v>67</v>
@@ -2714,13 +2714,13 @@
         <v>22</v>
       </c>
       <c r="B126">
-        <v>103.2714544255207</v>
+        <v>85.4927219413932</v>
       </c>
       <c r="C126">
-        <v>103.1831907722486</v>
+        <v>85.41641135742789</v>
       </c>
       <c r="D126">
-        <v>0.08826365327203689</v>
+        <v>0.07631058396530932</v>
       </c>
       <c r="E126" t="s">
         <v>68</v>
@@ -2731,13 +2731,13 @@
         <v>22</v>
       </c>
       <c r="B127">
-        <v>101.876563743982</v>
+        <v>97.50758148668559</v>
       </c>
       <c r="C127">
-        <v>101.784097116044</v>
+        <v>97.42026012021527</v>
       </c>
       <c r="D127">
-        <v>0.09246662793799487</v>
+        <v>0.08732136647032007</v>
       </c>
       <c r="E127" t="s">
         <v>69</v>
@@ -2748,13 +2748,13 @@
         <v>23</v>
       </c>
       <c r="B128">
-        <v>102.4140746993041</v>
+        <v>91.2233763934936</v>
       </c>
       <c r="C128">
-        <v>102.323620435305</v>
+        <v>91.14157330796969</v>
       </c>
       <c r="D128">
-        <v>0.09045426399903533</v>
+        <v>0.08180308552390159</v>
       </c>
       <c r="E128" t="s">
         <v>63</v>
@@ -2765,13 +2765,13 @@
         <v>23</v>
       </c>
       <c r="B129">
-        <v>102.6175611192371</v>
+        <v>83.31326464095062</v>
       </c>
       <c r="C129">
-        <v>102.5295603877825</v>
+        <v>83.23876996720584</v>
       </c>
       <c r="D129">
-        <v>0.08800073145458498</v>
+        <v>0.07449467374478047</v>
       </c>
       <c r="E129" t="s">
         <v>64</v>
@@ -2782,13 +2782,13 @@
         <v>23</v>
       </c>
       <c r="B130">
-        <v>102.4335821809334</v>
+        <v>99.91487487478186</v>
       </c>
       <c r="C130">
-        <v>102.3403916079477</v>
+        <v>99.82503595455172</v>
       </c>
       <c r="D130">
-        <v>0.09319057298570499</v>
+        <v>0.08983892023013595</v>
       </c>
       <c r="E130" t="s">
         <v>65</v>
@@ -2799,13 +2799,13 @@
         <v>23</v>
       </c>
       <c r="B131">
-        <v>101.8507953432165</v>
+        <v>92.75807495766831</v>
       </c>
       <c r="C131">
-        <v>101.7595407066255</v>
+        <v>92.67488917980671</v>
       </c>
       <c r="D131">
-        <v>0.09125463659098898</v>
+        <v>0.0831857778616012</v>
       </c>
       <c r="E131" t="s">
         <v>66</v>
@@ -2816,13 +2816,13 @@
         <v>23</v>
       </c>
       <c r="B132">
-        <v>103.1126080527711</v>
+        <v>88.06235784183525</v>
       </c>
       <c r="C132">
-        <v>103.0233662114269</v>
+        <v>87.98344052788859</v>
       </c>
       <c r="D132">
-        <v>0.08924184134411917</v>
+        <v>0.07891731394666124</v>
       </c>
       <c r="E132" t="s">
         <v>67</v>
@@ -2833,13 +2833,13 @@
         <v>23</v>
       </c>
       <c r="B133">
-        <v>103.1473430183639</v>
+        <v>85.4123716239386</v>
       </c>
       <c r="C133">
-        <v>103.0588942667672</v>
+        <v>85.33590531201416</v>
       </c>
       <c r="D133">
-        <v>0.08844875159674359</v>
+        <v>0.07646631192443465</v>
       </c>
       <c r="E133" t="s">
         <v>68</v>
@@ -2850,13 +2850,13 @@
         <v>23</v>
       </c>
       <c r="B134">
-        <v>101.8249290652489</v>
+        <v>97.43968579297501</v>
       </c>
       <c r="C134">
-        <v>101.7322579309781</v>
+        <v>97.35217003628092</v>
       </c>
       <c r="D134">
-        <v>0.09267113427078755</v>
+        <v>0.08751575669408851</v>
       </c>
       <c r="E134" t="s">
         <v>69</v>
@@ -2867,13 +2867,13 @@
         <v>24</v>
       </c>
       <c r="B135">
-        <v>104.3507350405985</v>
+        <v>97.36265798951685</v>
       </c>
       <c r="C135">
-        <v>104.2804502711753</v>
+        <v>97.29722062103914</v>
       </c>
       <c r="D135">
-        <v>0.07028476942326733</v>
+        <v>0.06543736847770276</v>
       </c>
       <c r="E135" t="s">
         <v>63</v>
@@ -2884,13 +2884,13 @@
         <v>24</v>
       </c>
       <c r="B136">
-        <v>105.1559611687937</v>
+        <v>92.06350190684641</v>
       </c>
       <c r="C136">
-        <v>105.0861560935237</v>
+        <v>92.0016913380222</v>
       </c>
       <c r="D136">
-        <v>0.06980507527001123</v>
+        <v>0.06181056882421387</v>
       </c>
       <c r="E136" t="s">
         <v>64</v>
@@ -2901,13 +2901,13 @@
         <v>24</v>
       </c>
       <c r="B137">
-        <v>103.584472676976</v>
+        <v>102.9739067916901</v>
       </c>
       <c r="C137">
-        <v>103.5136643032324</v>
+        <v>102.9046273091696</v>
       </c>
       <c r="D137">
-        <v>0.07080837374356008</v>
+        <v>0.06927948252048566</v>
       </c>
       <c r="E137" t="s">
         <v>65</v>
@@ -2918,13 +2918,13 @@
         <v>24</v>
       </c>
       <c r="B138">
-        <v>103.9004943042871</v>
+        <v>99.54917259078626</v>
       </c>
       <c r="C138">
-        <v>103.8299102691146</v>
+        <v>99.48225199018705</v>
       </c>
       <c r="D138">
-        <v>0.07058403517248735</v>
+        <v>0.06692060059920379</v>
       </c>
       <c r="E138" t="s">
         <v>66</v>
@@ -2935,13 +2935,13 @@
         <v>24</v>
       </c>
       <c r="B139">
-        <v>104.9945122830247</v>
+        <v>94.12114404978661</v>
       </c>
       <c r="C139">
-        <v>104.9246009240009</v>
+        <v>94.05791200236007</v>
       </c>
       <c r="D139">
-        <v>0.06991135902374879</v>
+        <v>0.06323204742653843</v>
       </c>
       <c r="E139" t="s">
         <v>67</v>
@@ -2952,13 +2952,13 @@
         <v>24</v>
       </c>
       <c r="B140">
-        <v>105.2360194841764</v>
+        <v>92.432403777673</v>
       </c>
       <c r="C140">
-        <v>105.1662591172353</v>
+        <v>92.3703284949944</v>
       </c>
       <c r="D140">
-        <v>0.06976036694116772</v>
+        <v>0.06207528267860596</v>
       </c>
       <c r="E140" t="s">
         <v>68</v>
@@ -2969,13 +2969,13 @@
         <v>24</v>
       </c>
       <c r="B141">
-        <v>103.4909611943969</v>
+        <v>102.5597969437173</v>
       </c>
       <c r="C141">
-        <v>103.4201094593854</v>
+        <v>102.4908140007436</v>
       </c>
       <c r="D141">
-        <v>0.07085173501151587</v>
+        <v>0.06898294297366192</v>
       </c>
       <c r="E141" t="s">
         <v>69</v>
@@ -2986,13 +2986,13 @@
         <v>25</v>
       </c>
       <c r="B142">
-        <v>104.1383478355649</v>
+        <v>104.147771323011</v>
       </c>
       <c r="C142">
-        <v>105.1411904335369</v>
+        <v>105.1521606771947</v>
       </c>
       <c r="D142">
-        <v>-1.002842597971977</v>
+        <v>-1.004389354183729</v>
       </c>
       <c r="E142" t="s">
         <v>63</v>
@@ -3003,13 +3003,13 @@
         <v>25</v>
       </c>
       <c r="B143">
-        <v>83.80602452163981</v>
+        <v>83.8145234874172</v>
       </c>
       <c r="C143">
-        <v>83.70355322444031</v>
+        <v>83.71204149443503</v>
       </c>
       <c r="D143">
-        <v>0.1024712971995001</v>
+        <v>0.1024819929821774</v>
       </c>
       <c r="E143" t="s">
         <v>64</v>
@@ -3020,13 +3020,13 @@
         <v>25</v>
       </c>
       <c r="B144">
-        <v>116.3234621141064</v>
+        <v>116.3320685192221</v>
       </c>
       <c r="C144">
-        <v>133.4712790041389</v>
+        <v>133.4855542927207</v>
       </c>
       <c r="D144">
-        <v>-17.14781689003253</v>
+        <v>-17.15348577349859</v>
       </c>
       <c r="E144" t="s">
         <v>65</v>
@@ -3037,13 +3037,13 @@
         <v>25</v>
       </c>
       <c r="B145">
-        <v>97.8047485808525</v>
+        <v>97.81474237675549</v>
       </c>
       <c r="C145">
-        <v>97.70481989202449</v>
+        <v>97.71486564988814</v>
       </c>
       <c r="D145">
-        <v>0.09992868882801531</v>
+        <v>0.09987672686735038</v>
       </c>
       <c r="E145" t="s">
         <v>66</v>
@@ -3054,13 +3054,13 @@
         <v>25</v>
       </c>
       <c r="B146">
-        <v>102.2980982463725</v>
+        <v>102.3058948620488</v>
       </c>
       <c r="C146">
-        <v>108.2421207594155</v>
+        <v>108.2535141248661</v>
       </c>
       <c r="D146">
-        <v>-5.944022513043009</v>
+        <v>-5.947619262817383</v>
       </c>
       <c r="E146" t="s">
         <v>67</v>
@@ -3071,13 +3071,13 @@
         <v>25</v>
       </c>
       <c r="B147">
-        <v>97.51679529015789</v>
+        <v>97.52558993793478</v>
       </c>
       <c r="C147">
-        <v>99.06942163879438</v>
+        <v>99.07974236843837</v>
       </c>
       <c r="D147">
-        <v>-1.552626348636494</v>
+        <v>-1.554152430503592</v>
       </c>
       <c r="E147" t="s">
         <v>68</v>
@@ -3088,13 +3088,13 @@
         <v>25</v>
       </c>
       <c r="B148">
-        <v>110.4073853825261</v>
+        <v>110.417367758813</v>
       </c>
       <c r="C148">
-        <v>111.5977095552461</v>
+        <v>111.6093708510414</v>
       </c>
       <c r="D148">
-        <v>-1.190324172720011</v>
+        <v>-1.192003092228333</v>
       </c>
       <c r="E148" t="s">
         <v>69</v>
@@ -3105,13 +3105,13 @@
         <v>26</v>
       </c>
       <c r="B149">
-        <v>104.4102654916629</v>
+        <v>86.92124127858565</v>
       </c>
       <c r="C149">
-        <v>104.2975535277135</v>
+        <v>86.82326312635855</v>
       </c>
       <c r="D149">
-        <v>0.1127119639494083</v>
+        <v>0.09797815222709971</v>
       </c>
       <c r="E149" t="s">
         <v>63</v>
@@ -3122,13 +3122,13 @@
         <v>26</v>
       </c>
       <c r="B150">
-        <v>104.0139088705514</v>
+        <v>75.01159072882399</v>
       </c>
       <c r="C150">
-        <v>103.9079239567337</v>
+        <v>74.92789141620285</v>
       </c>
       <c r="D150">
-        <v>0.1059849138177356</v>
+        <v>0.08369931262113539</v>
       </c>
       <c r="E150" t="s">
         <v>64</v>
@@ -3139,13 +3139,13 @@
         <v>26</v>
       </c>
       <c r="B151">
-        <v>105.6395785308202</v>
+        <v>100.8895759068823</v>
       </c>
       <c r="C151">
-        <v>105.5189273180302</v>
+        <v>100.7748317904294</v>
       </c>
       <c r="D151">
-        <v>0.1206512127900652</v>
+        <v>0.1147441164529397</v>
       </c>
       <c r="E151" t="s">
         <v>65</v>
@@ -3156,13 +3156,13 @@
         <v>26</v>
       </c>
       <c r="B152">
-        <v>102.7694033553193</v>
+        <v>85.96046271672296</v>
       </c>
       <c r="C152">
-        <v>102.656134878459</v>
+        <v>85.86372331766567</v>
       </c>
       <c r="D152">
-        <v>0.1132684768602843</v>
+        <v>0.09673939905728446</v>
       </c>
       <c r="E152" t="s">
         <v>66</v>
@@ -3173,13 +3173,13 @@
         <v>26</v>
       </c>
       <c r="B153">
-        <v>106.1835106747425</v>
+        <v>85.32664861938335</v>
       </c>
       <c r="C153">
-        <v>106.0725325691629</v>
+        <v>85.23049714258354</v>
       </c>
       <c r="D153">
-        <v>0.110978105579548</v>
+        <v>0.09615147679980396</v>
       </c>
       <c r="E153" t="s">
         <v>67</v>
@@ -3190,13 +3190,13 @@
         <v>26</v>
       </c>
       <c r="B154">
-        <v>105.9358623015307</v>
+        <v>80.98994465457615</v>
       </c>
       <c r="C154">
-        <v>105.8271920706346</v>
+        <v>80.89900034277123</v>
       </c>
       <c r="D154">
-        <v>0.108670230896152</v>
+        <v>0.09094431180491824</v>
       </c>
       <c r="E154" t="s">
         <v>68</v>
@@ -3207,13 +3207,13 @@
         <v>26</v>
       </c>
       <c r="B155">
-        <v>103.2692266182532</v>
+        <v>93.31047777482208</v>
       </c>
       <c r="C155">
-        <v>103.1519237721811</v>
+        <v>93.20491656666901</v>
       </c>
       <c r="D155">
-        <v>0.1173028460721497</v>
+        <v>0.1055612081530626</v>
       </c>
       <c r="E155" t="s">
         <v>69</v>
@@ -3224,13 +3224,13 @@
         <v>27</v>
       </c>
       <c r="B156">
-        <v>105.6049252129322</v>
+        <v>105.6142221069481</v>
       </c>
       <c r="C156">
-        <v>106.7187951710539</v>
+        <v>106.7297522461004</v>
       </c>
       <c r="D156">
-        <v>-1.113869958121725</v>
+        <v>-1.115530139152284</v>
       </c>
       <c r="E156" t="s">
         <v>63</v>
@@ -3241,13 +3241,13 @@
         <v>27</v>
       </c>
       <c r="B157">
-        <v>85.6613272638338</v>
+        <v>85.66985557630152</v>
       </c>
       <c r="C157">
-        <v>85.55855731867103</v>
+        <v>85.56707651828657</v>
       </c>
       <c r="D157">
-        <v>0.1027699451627626</v>
+        <v>0.1027790580149457</v>
       </c>
       <c r="E157" t="s">
         <v>64</v>
@@ -3258,13 +3258,13 @@
         <v>27</v>
       </c>
       <c r="B158">
-        <v>116.9036140281033</v>
+        <v>116.9118440911462</v>
       </c>
       <c r="C158">
-        <v>134.5215743901397</v>
+        <v>134.5357587031455</v>
       </c>
       <c r="D158">
-        <v>-17.6179603620364</v>
+        <v>-17.62391461199925</v>
       </c>
       <c r="E158" t="s">
         <v>65</v>
@@ -3275,13 +3275,13 @@
         <v>27</v>
       </c>
       <c r="B159">
-        <v>99.67227316684985</v>
+        <v>99.68228539671588</v>
       </c>
       <c r="C159">
-        <v>99.58081640647698</v>
+        <v>99.5908882128869</v>
       </c>
       <c r="D159">
-        <v>0.09145676037286421</v>
+        <v>0.0913971838289882</v>
       </c>
       <c r="E159" t="s">
         <v>66</v>
@@ -3292,13 +3292,13 @@
         <v>27</v>
       </c>
       <c r="B160">
-        <v>103.5424377144012</v>
+        <v>103.5499635993058</v>
       </c>
       <c r="C160">
-        <v>109.5593412227191</v>
+        <v>109.5706889355631</v>
       </c>
       <c r="D160">
-        <v>-6.01690350831791</v>
+        <v>-6.0207253362573</v>
       </c>
       <c r="E160" t="s">
         <v>67</v>
@@ -3309,13 +3309,13 @@
         <v>27</v>
       </c>
       <c r="B161">
-        <v>99.00617887021099</v>
+        <v>99.01485782473394</v>
       </c>
       <c r="C161">
-        <v>100.5872470905939</v>
+        <v>100.5975509989438</v>
       </c>
       <c r="D161">
-        <v>-1.581068220382903</v>
+        <v>-1.582693174209894</v>
       </c>
       <c r="E161" t="s">
         <v>68</v>
@@ -3326,13 +3326,13 @@
         <v>27</v>
       </c>
       <c r="B162">
-        <v>111.841950901682</v>
+        <v>111.8517950546726</v>
       </c>
       <c r="C162">
-        <v>113.240873819161</v>
+        <v>113.2525261665448</v>
       </c>
       <c r="D162">
-        <v>-1.398922917478913</v>
+        <v>-1.400731111872176</v>
       </c>
       <c r="E162" t="s">
         <v>69</v>
@@ -3343,13 +3343,13 @@
         <v>28</v>
       </c>
       <c r="B163">
-        <v>107.1079622228388</v>
+        <v>107.1131616707679</v>
       </c>
       <c r="C163">
-        <v>107.0449820681002</v>
+        <v>107.0501783706839</v>
       </c>
       <c r="D163">
-        <v>0.06298015473855401</v>
+        <v>0.06298330008401365</v>
       </c>
       <c r="E163" t="s">
         <v>63</v>
@@ -3360,13 +3360,13 @@
         <v>28</v>
       </c>
       <c r="B164">
-        <v>102.2492162480294</v>
+        <v>102.2541723235569</v>
       </c>
       <c r="C164">
-        <v>102.189184015697</v>
+        <v>102.1941370949359</v>
       </c>
       <c r="D164">
-        <v>0.06003223233238941</v>
+        <v>0.06003522862096133</v>
       </c>
       <c r="E164" t="s">
         <v>64</v>
@@ -3377,13 +3377,13 @@
         <v>28</v>
       </c>
       <c r="B165">
-        <v>112.206253924484</v>
+        <v>112.2117088705904</v>
       </c>
       <c r="C165">
-        <v>112.1401789703836</v>
+        <v>112.1456306146309</v>
       </c>
       <c r="D165">
-        <v>0.06607495410041508</v>
+        <v>0.06607825595955319</v>
       </c>
       <c r="E165" t="s">
         <v>65</v>
@@ -3394,13 +3394,13 @@
         <v>28</v>
       </c>
       <c r="B166">
-        <v>109.4199886240067</v>
+        <v>109.4253028171975</v>
       </c>
       <c r="C166">
-        <v>109.3556185806588</v>
+        <v>109.360929558478</v>
       </c>
       <c r="D166">
-        <v>0.06437004334789265</v>
+        <v>0.06437325871952737</v>
       </c>
       <c r="E166" t="s">
         <v>66</v>
@@ -3411,13 +3411,13 @@
         <v>28</v>
       </c>
       <c r="B167">
-        <v>103.8345139743774</v>
+        <v>103.8395505328191</v>
       </c>
       <c r="C167">
-        <v>103.7735068698799</v>
+        <v>103.7785403824858</v>
       </c>
       <c r="D167">
-        <v>0.06100710449744895</v>
+        <v>0.06101015033327428</v>
       </c>
       <c r="E167" t="s">
         <v>67</v>
@@ -3428,13 +3428,13 @@
         <v>28</v>
       </c>
       <c r="B168">
-        <v>102.3100056930851</v>
+        <v>102.3149658145373</v>
       </c>
       <c r="C168">
-        <v>102.2499244548089</v>
+        <v>102.2548815772578</v>
       </c>
       <c r="D168">
-        <v>0.06008123827622569</v>
+        <v>0.06008423727948298</v>
       </c>
       <c r="E168" t="s">
         <v>68</v>
@@ -3445,13 +3445,13 @@
         <v>28</v>
       </c>
       <c r="B169">
-        <v>112.1372619479288</v>
+        <v>112.1427123976534</v>
       </c>
       <c r="C169">
-        <v>112.0712414560099</v>
+        <v>112.0766886068753</v>
       </c>
       <c r="D169">
-        <v>0.06602049191890558</v>
+        <v>0.06602379077817488</v>
       </c>
       <c r="E169" t="s">
         <v>69</v>
@@ -3462,13 +3462,13 @@
         <v>29</v>
       </c>
       <c r="B170">
-        <v>104.9579119843815</v>
+        <v>104.967263841573</v>
       </c>
       <c r="C170">
-        <v>106.0207505520693</v>
+        <v>106.0317157059055</v>
       </c>
       <c r="D170">
-        <v>-1.062838567687791</v>
+        <v>-1.064451864332497</v>
       </c>
       <c r="E170" t="s">
         <v>63</v>
@@ -3479,13 +3479,13 @@
         <v>29</v>
       </c>
       <c r="B171">
-        <v>84.83976685403302</v>
+        <v>84.8482852329962</v>
       </c>
       <c r="C171">
-        <v>84.73710160533427</v>
+        <v>84.74560947083569</v>
       </c>
       <c r="D171">
-        <v>0.1026652486987416</v>
+        <v>0.1026757621605157</v>
       </c>
       <c r="E171" t="s">
         <v>64</v>
@@ -3496,13 +3496,13 @@
         <v>29</v>
       </c>
       <c r="B172">
-        <v>116.6590410671116</v>
+        <v>116.6674483343186</v>
       </c>
       <c r="C172">
-        <v>134.0558448258811</v>
+        <v>134.0700713170076</v>
       </c>
       <c r="D172">
-        <v>-17.39680375876952</v>
+        <v>-17.40262298268892</v>
       </c>
       <c r="E172" t="s">
         <v>65</v>
@@ -3513,13 +3513,13 @@
         <v>29</v>
       </c>
       <c r="B173">
-        <v>98.85102403100562</v>
+        <v>98.86101965648449</v>
       </c>
       <c r="C173">
-        <v>98.75425653050213</v>
+        <v>98.76431936783334</v>
       </c>
       <c r="D173">
-        <v>0.09676750050348915</v>
+        <v>0.09670028865114944</v>
       </c>
       <c r="E173" t="s">
         <v>66</v>
@@ -3530,13 +3530,13 @@
         <v>29</v>
       </c>
       <c r="B174">
-        <v>102.9848632679722</v>
+        <v>102.9925321930304</v>
       </c>
       <c r="C174">
-        <v>108.9724093969097</v>
+        <v>108.9837792179766</v>
       </c>
       <c r="D174">
-        <v>-5.987546128937495</v>
+        <v>-5.991247024946233</v>
       </c>
       <c r="E174" t="s">
         <v>67</v>
@@ -3547,13 +3547,13 @@
         <v>29</v>
       </c>
       <c r="B175">
-        <v>98.34274012086618</v>
+        <v>98.35146904475539</v>
       </c>
       <c r="C175">
-        <v>99.9123383882679</v>
+        <v>99.92265180683195</v>
       </c>
       <c r="D175">
-        <v>-1.569598267401716</v>
+        <v>-1.57118276207656</v>
       </c>
       <c r="E175" t="s">
         <v>68</v>
@@ -3564,13 +3564,13 @@
         <v>29</v>
       </c>
       <c r="B176">
-        <v>111.2159499552103</v>
+        <v>111.2258543834898</v>
       </c>
       <c r="C176">
-        <v>112.5173183939743</v>
+        <v>112.5289771540084</v>
       </c>
       <c r="D176">
-        <v>-1.301368438763916</v>
+        <v>-1.303122770518556</v>
       </c>
       <c r="E176" t="s">
         <v>69</v>
@@ -3581,13 +3581,13 @@
         <v>30</v>
       </c>
       <c r="B177">
-        <v>105.4528327887368</v>
+        <v>105.4621442138925</v>
       </c>
       <c r="C177">
-        <v>106.5547324052203</v>
+        <v>106.5656917394603</v>
       </c>
       <c r="D177">
-        <v>-1.101899616483422</v>
+        <v>-1.103547525567819</v>
       </c>
       <c r="E177" t="s">
         <v>63</v>
@@ -3598,13 +3598,13 @@
         <v>30</v>
       </c>
       <c r="B178">
-        <v>85.46608841971141</v>
+        <v>85.47461408241288</v>
       </c>
       <c r="C178">
-        <v>85.36334274023008</v>
+        <v>85.37185930575104</v>
       </c>
       <c r="D178">
-        <v>0.1027456794813304</v>
+        <v>0.1027547766618397</v>
       </c>
       <c r="E178" t="s">
         <v>64</v>
@@ -3615,13 +3615,13 @@
         <v>30</v>
       </c>
       <c r="B179">
-        <v>116.8462131491031</v>
+        <v>116.854484600007</v>
       </c>
       <c r="C179">
-        <v>134.415906177119</v>
+        <v>134.4301013172646</v>
       </c>
       <c r="D179">
-        <v>-17.56969302801591</v>
+        <v>-17.57561671725766</v>
       </c>
       <c r="E179" t="s">
         <v>65</v>
@@ -3632,13 +3632,13 @@
         <v>30</v>
       </c>
       <c r="B180">
-        <v>99.47708336541847</v>
+        <v>99.48709370554194</v>
       </c>
       <c r="C180">
-        <v>99.38473078390709</v>
+        <v>99.3948005910128</v>
       </c>
       <c r="D180">
-        <v>0.09235258151137771</v>
+        <v>0.09229311452914146</v>
       </c>
       <c r="E180" t="s">
         <v>66</v>
@@ -3649,13 +3649,13 @@
         <v>30</v>
       </c>
       <c r="B181">
-        <v>103.4122869434186</v>
+        <v>103.4198430120148</v>
       </c>
       <c r="C181">
-        <v>109.4228292017821</v>
+        <v>109.4341826623514</v>
       </c>
       <c r="D181">
-        <v>-6.010542258363444</v>
+        <v>-6.014339650336623</v>
       </c>
       <c r="E181" t="s">
         <v>67</v>
@@ -3666,13 +3666,13 @@
         <v>30</v>
       </c>
       <c r="B182">
-        <v>98.85015245399266</v>
+        <v>98.85884467672408</v>
       </c>
       <c r="C182">
-        <v>100.4286626064006</v>
+        <v>100.4389691020234</v>
       </c>
       <c r="D182">
-        <v>-1.578510152407972</v>
+        <v>-1.580124425299374</v>
       </c>
       <c r="E182" t="s">
         <v>68</v>
@@ -3683,13 +3683,13 @@
         <v>30</v>
       </c>
       <c r="B183">
-        <v>111.6947923733483</v>
+        <v>111.7046523877544</v>
       </c>
       <c r="C183">
-        <v>113.0707656466028</v>
+        <v>113.0824198701634</v>
       </c>
       <c r="D183">
-        <v>-1.375973273254488</v>
+        <v>-1.377767482408984</v>
       </c>
       <c r="E183" t="s">
         <v>69</v>
@@ -3700,13 +3700,13 @@
         <v>31</v>
       </c>
       <c r="B184">
-        <v>105.4988639990026</v>
+        <v>105.5081683426393</v>
       </c>
       <c r="C184">
-        <v>106.6066999572787</v>
+        <v>106.6176570197133</v>
       </c>
       <c r="D184">
-        <v>-1.10783595827607</v>
+        <v>-1.109488677073998</v>
       </c>
       <c r="E184" t="s">
         <v>63</v>
@@ -3717,13 +3717,13 @@
         <v>31</v>
       </c>
       <c r="B185">
-        <v>85.54093804204811</v>
+        <v>85.549464957738</v>
       </c>
       <c r="C185">
-        <v>85.43818731043199</v>
+        <v>85.44670512285276</v>
       </c>
       <c r="D185">
-        <v>0.1027507316161262</v>
+        <v>0.1027598348852337</v>
       </c>
       <c r="E185" t="s">
         <v>64</v>
@@ -3734,13 +3734,13 @@
         <v>31</v>
       </c>
       <c r="B186">
-        <v>116.8491507728496</v>
+        <v>116.8574040311822</v>
       </c>
       <c r="C186">
-        <v>134.425272563136</v>
+        <v>134.4394592516861</v>
       </c>
       <c r="D186">
-        <v>-17.57612179028634</v>
+        <v>-17.58205522050382</v>
       </c>
       <c r="E186" t="s">
         <v>65</v>
@@ -3751,13 +3751,13 @@
         <v>31</v>
       </c>
       <c r="B187">
-        <v>99.55102220989978</v>
+        <v>99.56103328646149</v>
       </c>
       <c r="C187">
-        <v>99.45924986741812</v>
+        <v>99.46932046003782</v>
       </c>
       <c r="D187">
-        <v>0.09177234248166144</v>
+        <v>0.09171282642367373</v>
       </c>
       <c r="E187" t="s">
         <v>66</v>
@@ -3768,13 +3768,13 @@
         <v>31</v>
       </c>
       <c r="B188">
-        <v>103.4469867216055</v>
+        <v>103.4545293072684</v>
       </c>
       <c r="C188">
-        <v>109.4555301238295</v>
+        <v>109.4668788049111</v>
       </c>
       <c r="D188">
-        <v>-6.008543402224021</v>
+        <v>-6.012349497642717</v>
       </c>
       <c r="E188" t="s">
         <v>67</v>
@@ -3785,13 +3785,13 @@
         <v>31</v>
       </c>
       <c r="B189">
-        <v>98.89768078497382</v>
+        <v>98.90636644182156</v>
       </c>
       <c r="C189">
-        <v>100.4774362827739</v>
+        <v>100.487740280206</v>
       </c>
       <c r="D189">
-        <v>-1.579755497800051</v>
+        <v>-1.581373838384408</v>
       </c>
       <c r="E189" t="s">
         <v>68</v>
@@ -3802,13 +3802,13 @@
         <v>31</v>
       </c>
       <c r="B190">
-        <v>111.7391941380343</v>
+        <v>111.7490465777041</v>
       </c>
       <c r="C190">
-        <v>113.1263110717645</v>
+        <v>113.1379632883613</v>
       </c>
       <c r="D190">
-        <v>-1.387116933730226</v>
+        <v>-1.388916710657156</v>
       </c>
       <c r="E190" t="s">
         <v>69</v>
@@ -3819,13 +3819,13 @@
         <v>32</v>
       </c>
       <c r="B191">
-        <v>105.1226887835173</v>
+        <v>105.1302110875339</v>
       </c>
       <c r="C191">
-        <v>106.9530735360714</v>
+        <v>106.9638325329286</v>
       </c>
       <c r="D191">
-        <v>-1.830384752554011</v>
+        <v>-1.833621445394769</v>
       </c>
       <c r="E191" t="s">
         <v>63</v>
@@ -3836,13 +3836,13 @@
         <v>32</v>
       </c>
       <c r="B192">
-        <v>87.69407582018482</v>
+        <v>87.70268311615857</v>
       </c>
       <c r="C192">
-        <v>87.5902948695486</v>
+        <v>87.59889207940721</v>
       </c>
       <c r="D192">
-        <v>0.1037809506362208</v>
+        <v>0.1037910367513604</v>
       </c>
       <c r="E192" t="s">
         <v>64</v>
@@ -3853,13 +3853,13 @@
         <v>32</v>
       </c>
       <c r="B193">
-        <v>111.8142326225407</v>
+        <v>111.8200577776951</v>
       </c>
       <c r="C193">
-        <v>131.5530801685402</v>
+        <v>131.5666028794049</v>
       </c>
       <c r="D193">
-        <v>-19.73884754599956</v>
+        <v>-19.74654510170986</v>
       </c>
       <c r="E193" t="s">
         <v>65</v>
@@ -3870,13 +3870,13 @@
         <v>32</v>
       </c>
       <c r="B194">
-        <v>101.572623329851</v>
+        <v>101.5823370950647</v>
       </c>
       <c r="C194">
-        <v>101.5795424552437</v>
+        <v>101.5896497111403</v>
       </c>
       <c r="D194">
-        <v>-0.006919125392641945</v>
+        <v>-0.007312616075523692</v>
       </c>
       <c r="E194" t="s">
         <v>66</v>
@@ -3887,13 +3887,13 @@
         <v>32</v>
       </c>
       <c r="B195">
-        <v>102.5719181382452</v>
+        <v>102.5779568251579</v>
       </c>
       <c r="C195">
-        <v>108.2919092714632</v>
+        <v>108.3028693171664</v>
       </c>
       <c r="D195">
-        <v>-5.719991133218016</v>
+        <v>-5.724912492008499</v>
       </c>
       <c r="E195" t="s">
         <v>67</v>
@@ -3904,13 +3904,13 @@
         <v>32</v>
       </c>
       <c r="B196">
-        <v>99.09608559752451</v>
+        <v>99.10392989273316</v>
       </c>
       <c r="C196">
-        <v>100.4711801887106</v>
+        <v>100.48126004358</v>
       </c>
       <c r="D196">
-        <v>-1.375094591186141</v>
+        <v>-1.377330150846802</v>
       </c>
       <c r="E196" t="s">
         <v>68</v>
@@ -3921,13 +3921,13 @@
         <v>32</v>
       </c>
       <c r="B197">
-        <v>110.5981593242575</v>
+        <v>110.6052674789529</v>
       </c>
       <c r="C197">
-        <v>113.8696459906438</v>
+        <v>113.8811304605333</v>
       </c>
       <c r="D197">
-        <v>-3.27148666638638</v>
+        <v>-3.27586298158036</v>
       </c>
       <c r="E197" t="s">
         <v>69</v>
@@ -3938,13 +3938,13 @@
         <v>33</v>
       </c>
       <c r="B198">
-        <v>100.2418787728176</v>
+        <v>100.2515543070265</v>
       </c>
       <c r="C198">
-        <v>100.2732036551172</v>
+        <v>100.2832570915276</v>
       </c>
       <c r="D198">
-        <v>-0.03132488229957175</v>
+        <v>-0.03170278450110686</v>
       </c>
       <c r="E198" t="s">
         <v>63</v>
@@ -3955,13 +3955,13 @@
         <v>33</v>
       </c>
       <c r="B199">
-        <v>82.40934090868309</v>
+        <v>82.41740329615506</v>
       </c>
       <c r="C199">
-        <v>82.31172005902241</v>
+        <v>82.31977195828469</v>
       </c>
       <c r="D199">
-        <v>0.09762084966068585</v>
+        <v>0.09763133787036793</v>
       </c>
       <c r="E199" t="s">
         <v>64</v>
@@ -3972,13 +3972,13 @@
         <v>33</v>
       </c>
       <c r="B200">
-        <v>109.8313208786433</v>
+        <v>109.836519360732</v>
       </c>
       <c r="C200">
-        <v>122.9806413572697</v>
+        <v>122.9932385081858</v>
       </c>
       <c r="D200">
-        <v>-13.14932047862639</v>
+        <v>-13.15671914745377</v>
       </c>
       <c r="E200" t="s">
         <v>65</v>
@@ -3989,13 +3989,13 @@
         <v>33</v>
       </c>
       <c r="B201">
-        <v>95.51730432285693</v>
+        <v>95.52677134609246</v>
       </c>
       <c r="C201">
-        <v>95.40719743340033</v>
+        <v>95.41666710912106</v>
       </c>
       <c r="D201">
-        <v>0.1101068894566026</v>
+        <v>0.1101042369713952</v>
       </c>
       <c r="E201" t="s">
         <v>66</v>
@@ -4006,13 +4006,13 @@
         <v>33</v>
       </c>
       <c r="B202">
-        <v>99.93961840980975</v>
+        <v>99.94735926771963</v>
       </c>
       <c r="C202">
-        <v>101.3708897454307</v>
+        <v>101.3811067153263</v>
       </c>
       <c r="D202">
-        <v>-1.431271335620906</v>
+        <v>-1.433747447606706</v>
       </c>
       <c r="E202" t="s">
         <v>67</v>
@@ -4023,13 +4023,13 @@
         <v>33</v>
       </c>
       <c r="B203">
-        <v>94.14350842000616</v>
+        <v>94.15255462091564</v>
       </c>
       <c r="C203">
-        <v>94.16117947857694</v>
+        <v>94.17058759547831</v>
       </c>
       <c r="D203">
-        <v>-0.01767105857078377</v>
+        <v>-0.01803297456267217</v>
       </c>
       <c r="E203" t="s">
         <v>68</v>
@@ -4040,13 +4040,13 @@
         <v>33</v>
       </c>
       <c r="B204">
-        <v>106.1477189528232</v>
+        <v>106.1568314761728</v>
       </c>
       <c r="C204">
-        <v>106.8019017849316</v>
+        <v>106.8126453136098</v>
       </c>
       <c r="D204">
-        <v>-0.6541828321084182</v>
+        <v>-0.6558138374370515</v>
       </c>
       <c r="E204" t="s">
         <v>69</v>
@@ -4057,13 +4057,13 @@
         <v>34</v>
       </c>
       <c r="B205">
-        <v>104.997605517938</v>
+        <v>105.0069591327968</v>
       </c>
       <c r="C205">
-        <v>106.0637142263577</v>
+        <v>106.0746793310802</v>
       </c>
       <c r="D205">
-        <v>-1.066108708419691</v>
+        <v>-1.067720198283425</v>
       </c>
       <c r="E205" t="s">
         <v>63</v>
@@ -4074,13 +4074,13 @@
         <v>34</v>
       </c>
       <c r="B206">
-        <v>84.88251149200511</v>
+        <v>84.89102830353021</v>
       </c>
       <c r="C206">
-        <v>84.77984738789677</v>
+        <v>84.78835514689908</v>
       </c>
       <c r="D206">
-        <v>0.1026641041083423</v>
+        <v>0.102673156631127</v>
       </c>
       <c r="E206" t="s">
         <v>64</v>
@@ -4091,13 +4091,13 @@
         <v>34</v>
       </c>
       <c r="B207">
-        <v>116.6745974682617</v>
+        <v>116.6829911337087</v>
       </c>
       <c r="C207">
-        <v>134.0992696216449</v>
+        <v>134.1134961530067</v>
       </c>
       <c r="D207">
-        <v>-17.42467215338323</v>
+        <v>-17.43050501929807</v>
       </c>
       <c r="E207" t="s">
         <v>65</v>
@@ -4108,13 +4108,13 @@
         <v>34</v>
       </c>
       <c r="B208">
-        <v>98.89192877167487</v>
+        <v>98.90193245836481</v>
       </c>
       <c r="C208">
-        <v>98.7968458202424</v>
+        <v>98.80690858268554</v>
       </c>
       <c r="D208">
-        <v>0.09508295143247381</v>
+        <v>0.09502387567927428</v>
       </c>
       <c r="E208" t="s">
         <v>66</v>
@@ -4125,13 +4125,13 @@
         <v>34</v>
       </c>
       <c r="B209">
-        <v>103.0254899050612</v>
+        <v>103.0331345620705</v>
       </c>
       <c r="C209">
-        <v>109.0156831508581</v>
+        <v>109.0270529366639</v>
       </c>
       <c r="D209">
-        <v>-5.990193245796974</v>
+        <v>-5.993918374593434</v>
       </c>
       <c r="E209" t="s">
         <v>67</v>
@@ -4142,13 +4142,13 @@
         <v>34</v>
       </c>
       <c r="B210">
-        <v>98.38526354751922</v>
+        <v>98.39399432116453</v>
       </c>
       <c r="C210">
-        <v>99.9554086672258</v>
+        <v>99.96572201587858</v>
       </c>
       <c r="D210">
-        <v>-1.570145119706581</v>
+        <v>-1.571727694714056</v>
       </c>
       <c r="E210" t="s">
         <v>68</v>
@@ -4159,13 +4159,13 @@
         <v>34</v>
       </c>
       <c r="B211">
-        <v>111.2521561826648</v>
+        <v>111.2620622309635</v>
       </c>
       <c r="C211">
-        <v>112.5601955071123</v>
+        <v>112.5718542436862</v>
       </c>
       <c r="D211">
-        <v>-1.308039324447421</v>
+        <v>-1.30979201272271</v>
       </c>
       <c r="E211" t="s">
         <v>69</v>
@@ -4176,13 +4176,13 @@
         <v>35</v>
       </c>
       <c r="B212">
-        <v>105.1491722647487</v>
+        <v>105.1585120376129</v>
       </c>
       <c r="C212">
-        <v>106.2271887439795</v>
+        <v>106.2381520859866</v>
       </c>
       <c r="D212">
-        <v>-1.07801647923074</v>
+        <v>-1.079640048373747</v>
       </c>
       <c r="E212" t="s">
         <v>63</v>
@@ -4193,13 +4193,13 @@
         <v>35</v>
       </c>
       <c r="B213">
-        <v>85.0766784882375</v>
+        <v>85.08519839485569</v>
       </c>
       <c r="C213">
-        <v>84.97398580293675</v>
+        <v>84.98249664266839</v>
       </c>
       <c r="D213">
-        <v>0.1026926853007524</v>
+        <v>0.1027017521873006</v>
       </c>
       <c r="E213" t="s">
         <v>64</v>
@@ -4210,13 +4210,13 @@
         <v>35</v>
       </c>
       <c r="B214">
-        <v>116.7317040193808</v>
+        <v>116.740057269207</v>
       </c>
       <c r="C214">
-        <v>134.2047492293683</v>
+        <v>134.2189654694051</v>
       </c>
       <c r="D214">
-        <v>-17.47304520998757</v>
+        <v>-17.47890820019815</v>
       </c>
       <c r="E214" t="s">
         <v>65</v>
@@ -4227,13 +4227,13 @@
         <v>35</v>
       </c>
       <c r="B215">
-        <v>99.08690757287691</v>
+        <v>99.0969136341155</v>
       </c>
       <c r="C215">
-        <v>98.99274153824337</v>
+        <v>99.00280681718971</v>
       </c>
       <c r="D215">
-        <v>0.09416603463354534</v>
+        <v>0.09410681692578748</v>
       </c>
       <c r="E215" t="s">
         <v>66</v>
@@ -4244,13 +4244,13 @@
         <v>35</v>
       </c>
       <c r="B216">
-        <v>103.1538154489844</v>
+        <v>103.1614308953446</v>
       </c>
       <c r="C216">
-        <v>109.1509978214199</v>
+        <v>109.1623623107847</v>
       </c>
       <c r="D216">
-        <v>-5.997182372435546</v>
+        <v>-6.000931415440135</v>
       </c>
       <c r="E216" t="s">
         <v>67</v>
@@ -4261,13 +4261,13 @@
         <v>35</v>
       </c>
       <c r="B217">
-        <v>98.53969432386062</v>
+        <v>98.54841244167834</v>
       </c>
       <c r="C217">
-        <v>100.1127415353614</v>
+        <v>100.1230527441903</v>
       </c>
       <c r="D217">
-        <v>-1.573047211500779</v>
+        <v>-1.574640302511924</v>
       </c>
       <c r="E217" t="s">
         <v>68</v>
@@ -4278,13 +4278,13 @@
         <v>35</v>
       </c>
       <c r="B218">
-        <v>111.3998949007002</v>
+        <v>111.409785847701</v>
       </c>
       <c r="C218">
-        <v>112.730422100051</v>
+        <v>112.7420795109943</v>
       </c>
       <c r="D218">
-        <v>-1.330527199350811</v>
+        <v>-1.332293663293314</v>
       </c>
       <c r="E218" t="s">
         <v>69</v>
@@ -4295,13 +4295,13 @@
         <v>36</v>
       </c>
       <c r="B219">
-        <v>104.1832137966851</v>
+        <v>104.1909162134904</v>
       </c>
       <c r="C219">
-        <v>105.901418558694</v>
+        <v>105.9121993854622</v>
       </c>
       <c r="D219">
-        <v>-1.718204762008924</v>
+        <v>-1.721283171971805</v>
       </c>
       <c r="E219" t="s">
         <v>63</v>
@@ -4312,13 +4312,13 @@
         <v>36</v>
       </c>
       <c r="B220">
-        <v>86.39731408808406</v>
+        <v>86.40590534634346</v>
       </c>
       <c r="C220">
-        <v>86.29378902549817</v>
+        <v>86.3023704296439</v>
       </c>
       <c r="D220">
-        <v>0.1035250625858879</v>
+        <v>0.1035349166995587</v>
       </c>
       <c r="E220" t="s">
         <v>64</v>
@@ -4329,13 +4329,13 @@
         <v>36</v>
       </c>
       <c r="B221">
-        <v>111.4285568509014</v>
+        <v>111.4347105174433</v>
       </c>
       <c r="C221">
-        <v>130.9236150342279</v>
+        <v>130.9372204946744</v>
       </c>
       <c r="D221">
-        <v>-19.49505818332655</v>
+        <v>-19.50250997723116</v>
       </c>
       <c r="E221" t="s">
         <v>65</v>
@@ -4346,13 +4346,13 @@
         <v>36</v>
       </c>
       <c r="B222">
-        <v>100.2973418086848</v>
+        <v>100.3072685546526</v>
       </c>
       <c r="C222">
-        <v>100.2749684723782</v>
+        <v>100.2850657030867</v>
       </c>
       <c r="D222">
-        <v>0.02237333630655769</v>
+        <v>0.0222028515658792</v>
       </c>
       <c r="E222" t="s">
         <v>66</v>
@@ -4363,13 +4363,13 @@
         <v>36</v>
       </c>
       <c r="B223">
-        <v>101.644865239721</v>
+        <v>101.6511616727377</v>
       </c>
       <c r="C223">
-        <v>107.4600838508705</v>
+        <v>107.4710918420468</v>
       </c>
       <c r="D223">
-        <v>-5.815218611149447</v>
+        <v>-5.819930169309075</v>
       </c>
       <c r="E223" t="s">
         <v>67</v>
@@ -4380,13 +4380,13 @@
         <v>36</v>
       </c>
       <c r="B224">
-        <v>98.06092566921488</v>
+        <v>98.06888120512849</v>
       </c>
       <c r="C224">
-        <v>99.49528268824609</v>
+        <v>99.50538995422433</v>
       </c>
       <c r="D224">
-        <v>-1.434357019031211</v>
+        <v>-1.436508749095836</v>
       </c>
       <c r="E224" t="s">
         <v>68</v>
@@ -4397,13 +4397,13 @@
         <v>36</v>
       </c>
       <c r="B225">
-        <v>109.803609637066</v>
+        <v>109.8117302328492</v>
       </c>
       <c r="C225">
-        <v>112.7332010098815</v>
+        <v>112.7447008231588</v>
       </c>
       <c r="D225">
-        <v>-2.929591372815494</v>
+        <v>-2.932970590309651</v>
       </c>
       <c r="E225" t="s">
         <v>69</v>
@@ -4414,13 +4414,13 @@
         <v>37</v>
       </c>
       <c r="B226">
-        <v>100.3765161161741</v>
+        <v>69.5211624520152</v>
       </c>
       <c r="C226">
-        <v>100.7995846244417</v>
+        <v>69.42839305339484</v>
       </c>
       <c r="D226">
-        <v>-0.4230685082676615</v>
+        <v>0.09276939862036215</v>
       </c>
       <c r="E226" t="s">
         <v>63</v>
@@ -4431,13 +4431,13 @@
         <v>37</v>
       </c>
       <c r="B227">
-        <v>97.53257676845587</v>
+        <v>51.71112742135696</v>
       </c>
       <c r="C227">
-        <v>97.56101242915429</v>
+        <v>51.64497462184339</v>
       </c>
       <c r="D227">
-        <v>-0.02843566069842041</v>
+        <v>0.06615279951356712</v>
       </c>
       <c r="E227" t="s">
         <v>64</v>
@@ -4448,13 +4448,13 @@
         <v>37</v>
       </c>
       <c r="B228">
-        <v>103.5468219082129</v>
+        <v>94.49575189677564</v>
       </c>
       <c r="C228">
-        <v>107.3030062938209</v>
+        <v>94.82085572175666</v>
       </c>
       <c r="D228">
-        <v>-3.756184385608023</v>
+        <v>-0.3251038249810136</v>
       </c>
       <c r="E228" t="s">
         <v>65</v>
@@ -4465,13 +4465,13 @@
         <v>37</v>
       </c>
       <c r="B229">
-        <v>92.28975015654859</v>
+        <v>60.83119129215958</v>
       </c>
       <c r="C229">
-        <v>92.20760021382283</v>
+        <v>60.7517405710337</v>
       </c>
       <c r="D229">
-        <v>0.08214994272576348</v>
+        <v>0.07945072112588036</v>
       </c>
       <c r="E229" t="s">
         <v>66</v>
@@ -4482,13 +4482,13 @@
         <v>37</v>
       </c>
       <c r="B230">
-        <v>105.1675170341382</v>
+        <v>74.89680560774693</v>
       </c>
       <c r="C230">
-        <v>109.9377591870332</v>
+        <v>74.81079810980947</v>
       </c>
       <c r="D230">
-        <v>-4.770242152894951</v>
+        <v>0.08600749793745877</v>
       </c>
       <c r="E230" t="s">
         <v>67</v>
@@ -4499,13 +4499,13 @@
         <v>37</v>
       </c>
       <c r="B231">
-        <v>104.2486417335563</v>
+        <v>66.3038835470357</v>
       </c>
       <c r="C231">
-        <v>106.8605766912061</v>
+        <v>66.21579876703787</v>
       </c>
       <c r="D231">
-        <v>-2.611934957649893</v>
+        <v>0.08808477999782838</v>
       </c>
       <c r="E231" t="s">
         <v>68</v>
@@ -4516,13 +4516,13 @@
         <v>37</v>
       </c>
       <c r="B232">
-        <v>94.82482468912521</v>
+        <v>72.90800248519692</v>
       </c>
       <c r="C232">
-        <v>94.89533289876225</v>
+        <v>72.81046065619869</v>
       </c>
       <c r="D232">
-        <v>-0.07050820963704041</v>
+        <v>0.09754182899823149</v>
       </c>
       <c r="E232" t="s">
         <v>69</v>
@@ -4533,13 +4533,13 @@
         <v>38</v>
       </c>
       <c r="B233">
-        <v>102.2294011072405</v>
+        <v>83.73547505724004</v>
       </c>
       <c r="C233">
-        <v>103.4721051204377</v>
+        <v>83.63313243644494</v>
       </c>
       <c r="D233">
-        <v>-1.242704013197269</v>
+        <v>0.102342620795099</v>
       </c>
       <c r="E233" t="s">
         <v>63</v>
@@ -4550,13 +4550,13 @@
         <v>38</v>
       </c>
       <c r="B234">
-        <v>100.1294989024095</v>
+        <v>69.13575119807403</v>
       </c>
       <c r="C234">
-        <v>100.4639509872304</v>
+        <v>69.05274122104353</v>
       </c>
       <c r="D234">
-        <v>-0.3344520848209243</v>
+        <v>0.08300997703049973</v>
       </c>
       <c r="E234" t="s">
         <v>64</v>
@@ -4567,13 +4567,13 @@
         <v>38</v>
       </c>
       <c r="B235">
-        <v>102.7737124671302</v>
+        <v>101.6212263440549</v>
       </c>
       <c r="C235">
-        <v>107.9456395983277</v>
+        <v>101.7332180292197</v>
       </c>
       <c r="D235">
-        <v>-5.17192713119745</v>
+        <v>-0.1119916851648668</v>
       </c>
       <c r="E235" t="s">
         <v>65</v>
@@ -4584,13 +4584,13 @@
         <v>38</v>
       </c>
       <c r="B236">
-        <v>100.0720819657586</v>
+        <v>80.2296467950093</v>
       </c>
       <c r="C236">
-        <v>100.7957183045757</v>
+        <v>80.13222919628015</v>
       </c>
       <c r="D236">
-        <v>-0.7236363388171156</v>
+        <v>0.09741759872915168</v>
       </c>
       <c r="E236" t="s">
         <v>66</v>
@@ -4601,13 +4601,13 @@
         <v>38</v>
       </c>
       <c r="B237">
-        <v>103.1222784383786</v>
+        <v>84.12560709515078</v>
       </c>
       <c r="C237">
-        <v>105.8210567232339</v>
+        <v>84.02247038036863</v>
       </c>
       <c r="D237">
-        <v>-2.698778284855237</v>
+        <v>0.1031367147821527</v>
       </c>
       <c r="E237" t="s">
         <v>67</v>
@@ -4618,13 +4618,13 @@
         <v>38</v>
       </c>
       <c r="B238">
-        <v>102.7096224719023</v>
+        <v>78.38674820609128</v>
       </c>
       <c r="C238">
-        <v>104.4253122015573</v>
+        <v>78.29124355059797</v>
       </c>
       <c r="D238">
-        <v>-1.715689729655011</v>
+        <v>0.09550465549331477</v>
       </c>
       <c r="E238" t="s">
         <v>68</v>
@@ -4635,13 +4635,13 @@
         <v>38</v>
       </c>
       <c r="B239">
-        <v>101.1431442537347</v>
+        <v>89.464151433053</v>
       </c>
       <c r="C239">
-        <v>102.8088700180732</v>
+        <v>89.35447572410071</v>
       </c>
       <c r="D239">
-        <v>-1.665725764338546</v>
+        <v>0.1096757089522953</v>
       </c>
       <c r="E239" t="s">
         <v>69</v>
@@ -4652,13 +4652,13 @@
         <v>39</v>
       </c>
       <c r="B240">
-        <v>97.55601889271624</v>
+        <v>70.63790164901228</v>
       </c>
       <c r="C240">
-        <v>97.58275756300439</v>
+        <v>70.54256654361656</v>
       </c>
       <c r="D240">
-        <v>-0.0267386702881538</v>
+        <v>0.09533510539571921</v>
       </c>
       <c r="E240" t="s">
         <v>63</v>
@@ -4669,13 +4669,13 @@
         <v>39</v>
       </c>
       <c r="B241">
-        <v>94.84486444141822</v>
+        <v>54.68523115930078</v>
       </c>
       <c r="C241">
-        <v>94.77773314685145</v>
+        <v>54.61274288582321</v>
       </c>
       <c r="D241">
-        <v>0.06713129456677791</v>
+        <v>0.07248827347757469</v>
       </c>
       <c r="E241" t="s">
         <v>64</v>
@@ -4686,13 +4686,13 @@
         <v>39</v>
       </c>
       <c r="B242">
-        <v>100.8298629328187</v>
+        <v>91.58829091431336</v>
       </c>
       <c r="C242">
-        <v>102.8026134956058</v>
+        <v>91.61473821705998</v>
       </c>
       <c r="D242">
-        <v>-1.972750562787098</v>
+        <v>-0.02644730274661811</v>
       </c>
       <c r="E242" t="s">
         <v>65</v>
@@ -4703,13 +4703,13 @@
         <v>39</v>
       </c>
       <c r="B243">
-        <v>92.81058407104159</v>
+        <v>64.60896664212814</v>
       </c>
       <c r="C243">
-        <v>92.74999291500882</v>
+        <v>64.52239660797866</v>
       </c>
       <c r="D243">
-        <v>0.06059115603277121</v>
+        <v>0.0865700341494744</v>
       </c>
       <c r="E243" t="s">
         <v>66</v>
@@ -4720,13 +4720,13 @@
         <v>39</v>
       </c>
       <c r="B244">
-        <v>101.3636407400726</v>
+        <v>73.42317205469483</v>
       </c>
       <c r="C244">
-        <v>102.5074589427751</v>
+        <v>73.32393071213056</v>
       </c>
       <c r="D244">
-        <v>-1.143818202702505</v>
+        <v>0.09924134256426953</v>
       </c>
       <c r="E244" t="s">
         <v>67</v>
@@ -4737,13 +4737,13 @@
         <v>39</v>
       </c>
       <c r="B245">
-        <v>100.1792437555197</v>
+        <v>66.62567225146984</v>
       </c>
       <c r="C245">
-        <v>100.6944853155229</v>
+        <v>66.53597192212874</v>
       </c>
       <c r="D245">
-        <v>-0.515241560003119</v>
+        <v>0.08970032934109895</v>
       </c>
       <c r="E245" t="s">
         <v>68</v>
@@ -4754,13 +4754,13 @@
         <v>39</v>
       </c>
       <c r="B246">
-        <v>94.69357251026149</v>
+        <v>74.90313934624881</v>
       </c>
       <c r="C246">
-        <v>94.76597534989432</v>
+        <v>74.801813003614</v>
       </c>
       <c r="D246">
-        <v>-0.07240283963282934</v>
+        <v>0.1013263426348061</v>
       </c>
       <c r="E246" t="s">
         <v>69</v>
@@ -4771,13 +4771,13 @@
         <v>40</v>
       </c>
       <c r="B247">
-        <v>98.69554597971941</v>
+        <v>72.71517592459269</v>
       </c>
       <c r="C247">
-        <v>98.62627252356684</v>
+        <v>72.62119483135234</v>
       </c>
       <c r="D247">
-        <v>0.06927345615257252</v>
+        <v>0.09398109324034465</v>
       </c>
       <c r="E247" t="s">
         <v>63</v>
@@ -4788,13 +4788,13 @@
         <v>40</v>
       </c>
       <c r="B248">
-        <v>96.16959395033481</v>
+        <v>56.84493795825251</v>
       </c>
       <c r="C248">
-        <v>96.08066487729739</v>
+        <v>56.77366417876913</v>
       </c>
       <c r="D248">
-        <v>0.08892907303741993</v>
+        <v>0.0712737794833771</v>
       </c>
       <c r="E248" t="s">
         <v>64</v>
@@ -4805,13 +4805,13 @@
         <v>40</v>
       </c>
       <c r="B249">
-        <v>102.3082554638168</v>
+        <v>93.80223458552783</v>
       </c>
       <c r="C249">
-        <v>103.1932290203828</v>
+        <v>93.71636173038152</v>
       </c>
       <c r="D249">
-        <v>-0.8849735565660666</v>
+        <v>0.08587285514630594</v>
       </c>
       <c r="E249" t="s">
         <v>65</v>
@@ -4822,13 +4822,13 @@
         <v>40</v>
       </c>
       <c r="B250">
-        <v>91.96551360846544</v>
+        <v>65.75216184914154</v>
       </c>
       <c r="C250">
-        <v>91.86180833463781</v>
+        <v>65.66844350574652</v>
       </c>
       <c r="D250">
-        <v>0.1037052738276287</v>
+        <v>0.08371834339502016</v>
       </c>
       <c r="E250" t="s">
         <v>66</v>
@@ -4839,13 +4839,13 @@
         <v>40</v>
       </c>
       <c r="B251">
-        <v>104.4442634447755</v>
+        <v>76.28188462386893</v>
       </c>
       <c r="C251">
-        <v>105.2882276776264</v>
+        <v>76.18263610195383</v>
       </c>
       <c r="D251">
-        <v>-0.8439642328509507</v>
+        <v>0.0992485219151007</v>
       </c>
       <c r="E251" t="s">
         <v>67</v>
@@ -4856,13 +4856,13 @@
         <v>40</v>
       </c>
       <c r="B252">
-        <v>102.4800823929831</v>
+        <v>68.73197074151751</v>
       </c>
       <c r="C252">
-        <v>102.7164549359843</v>
+        <v>68.64345535038358</v>
       </c>
       <c r="D252">
-        <v>-0.2363725430011669</v>
+        <v>0.08851539113393869</v>
       </c>
       <c r="E252" t="s">
         <v>68</v>
@@ -4873,13 +4873,13 @@
         <v>40</v>
       </c>
       <c r="B253">
-        <v>94.77463638637404</v>
+        <v>76.94402380264111</v>
       </c>
       <c r="C253">
-        <v>94.72695081600537</v>
+        <v>76.84423452828818</v>
       </c>
       <c r="D253">
-        <v>0.04768557036867094</v>
+        <v>0.09978927435292917</v>
       </c>
       <c r="E253" t="s">
         <v>69</v>
@@ -4890,13 +4890,13 @@
         <v>41</v>
       </c>
       <c r="B254">
-        <v>100.6256491097889</v>
+        <v>74.23200579750389</v>
       </c>
       <c r="C254">
-        <v>100.6360390583657</v>
+        <v>74.13592319475448</v>
       </c>
       <c r="D254">
-        <v>-0.0103899485768153</v>
+        <v>0.09608260274940505</v>
       </c>
       <c r="E254" t="s">
         <v>63</v>
@@ -4907,13 +4907,13 @@
         <v>41</v>
       </c>
       <c r="B255">
-        <v>99.04917259345407</v>
+        <v>58.25831391885705</v>
       </c>
       <c r="C255">
-        <v>98.96840155582525</v>
+        <v>58.18504705617319</v>
       </c>
       <c r="D255">
-        <v>0.08077103762882132</v>
+        <v>0.07326686268385885</v>
       </c>
       <c r="E255" t="s">
         <v>64</v>
@@ -4924,13 +4924,13 @@
         <v>41</v>
       </c>
       <c r="B256">
-        <v>102.5241231844777</v>
+        <v>95.13740757903042</v>
       </c>
       <c r="C256">
-        <v>104.5741784919224</v>
+        <v>95.17042496672528</v>
       </c>
       <c r="D256">
-        <v>-2.050055307444723</v>
+        <v>-0.03301738769485496</v>
       </c>
       <c r="E256" t="s">
         <v>65</v>
@@ -4941,13 +4941,13 @@
         <v>41</v>
       </c>
       <c r="B257">
-        <v>94.71726128149932</v>
+        <v>68.26325208400755</v>
       </c>
       <c r="C257">
-        <v>94.64703895360701</v>
+        <v>68.17581978053957</v>
       </c>
       <c r="D257">
-        <v>0.07022232789230998</v>
+        <v>0.08743230346797759</v>
       </c>
       <c r="E257" t="s">
         <v>66</v>
@@ -4958,13 +4958,13 @@
         <v>41</v>
       </c>
       <c r="B258">
-        <v>105.868815597866</v>
+        <v>76.94860453353823</v>
       </c>
       <c r="C258">
-        <v>106.9374892292422</v>
+        <v>76.84869158070948</v>
       </c>
       <c r="D258">
-        <v>-1.068673631376271</v>
+        <v>0.09991295282874546</v>
       </c>
       <c r="E258" t="s">
         <v>67</v>
@@ -4975,13 +4975,13 @@
         <v>41</v>
       </c>
       <c r="B259">
-        <v>105.0466189391316</v>
+        <v>70.17507407437597</v>
       </c>
       <c r="C259">
-        <v>105.4916986506749</v>
+        <v>70.0846796378579</v>
       </c>
       <c r="D259">
-        <v>-0.4450797115432721</v>
+        <v>0.09039443651806778</v>
       </c>
       <c r="E259" t="s">
         <v>68</v>
@@ -4992,13 +4992,13 @@
         <v>41</v>
       </c>
       <c r="B260">
-        <v>96.02025315965695</v>
+        <v>78.54505515660075</v>
       </c>
       <c r="C260">
-        <v>96.08539617565962</v>
+        <v>78.44292398439811</v>
       </c>
       <c r="D260">
-        <v>-0.06514301600267913</v>
+        <v>0.1021311722026468</v>
       </c>
       <c r="E260" t="s">
         <v>69</v>
@@ -5009,13 +5009,13 @@
         <v>42</v>
       </c>
       <c r="B261">
-        <v>99.45270691600022</v>
+        <v>73.03929466835368</v>
       </c>
       <c r="C261">
-        <v>99.44859746239956</v>
+        <v>72.94360526266836</v>
       </c>
       <c r="D261">
-        <v>0.004109453600662505</v>
+        <v>0.09568940568532014</v>
       </c>
       <c r="E261" t="s">
         <v>63</v>
@@ -5026,13 +5026,13 @@
         <v>42</v>
       </c>
       <c r="B262">
-        <v>97.54826870540779</v>
+        <v>56.96841047811881</v>
       </c>
       <c r="C262">
-        <v>97.46566660422596</v>
+        <v>56.89576665715194</v>
       </c>
       <c r="D262">
-        <v>0.08260210118183409</v>
+        <v>0.07264382096687427</v>
       </c>
       <c r="E262" t="s">
         <v>64</v>
@@ -5043,13 +5043,13 @@
         <v>42</v>
       </c>
       <c r="B263">
-        <v>101.8483636570298</v>
+        <v>94.20172728071479</v>
       </c>
       <c r="C263">
-        <v>103.7262934324435</v>
+        <v>94.22117876614473</v>
       </c>
       <c r="D263">
-        <v>-1.877929775413691</v>
+        <v>-0.01945148542993991</v>
       </c>
       <c r="E263" t="s">
         <v>65</v>
@@ -5060,13 +5060,13 @@
         <v>42</v>
       </c>
       <c r="B264">
-        <v>93.60063888169931</v>
+        <v>66.91772860809277</v>
       </c>
       <c r="C264">
-        <v>93.52104600042912</v>
+        <v>66.83097953712112</v>
       </c>
       <c r="D264">
-        <v>0.07959288127018738</v>
+        <v>0.08674907097164919</v>
       </c>
       <c r="E264" t="s">
         <v>66</v>
@@ -5077,13 +5077,13 @@
         <v>42</v>
       </c>
       <c r="B265">
-        <v>104.5772541298888</v>
+        <v>75.89737972053631</v>
       </c>
       <c r="C265">
-        <v>105.6296341809036</v>
+        <v>75.79766201640906</v>
       </c>
       <c r="D265">
-        <v>-1.052380051014765</v>
+        <v>0.09971770412724368</v>
       </c>
       <c r="E265" t="s">
         <v>67</v>
@@ -5094,13 +5094,13 @@
         <v>42</v>
       </c>
       <c r="B266">
-        <v>103.5924900772574</v>
+        <v>69.02462297827815</v>
       </c>
       <c r="C266">
-        <v>104.0276605327914</v>
+        <v>68.93455120574288</v>
       </c>
       <c r="D266">
-        <v>-0.4351704555340206</v>
+        <v>0.09007177253526777</v>
       </c>
       <c r="E266" t="s">
         <v>68</v>
@@ -5111,13 +5111,13 @@
         <v>42</v>
       </c>
       <c r="B267">
-        <v>95.08943150847577</v>
+        <v>77.30449868538994</v>
       </c>
       <c r="C267">
-        <v>95.1262775135523</v>
+        <v>77.20283768824427</v>
       </c>
       <c r="D267">
-        <v>-0.03684600507652647</v>
+        <v>0.1016609971456717</v>
       </c>
       <c r="E267" t="s">
         <v>69</v>
@@ -5128,13 +5128,13 @@
         <v>43</v>
       </c>
       <c r="B268">
-        <v>105.0469210890513</v>
+        <v>87.51195400482506</v>
       </c>
       <c r="C268">
-        <v>104.934854189452</v>
+        <v>87.41435981388619</v>
       </c>
       <c r="D268">
-        <v>0.1120668995993412</v>
+        <v>0.09759419093886379</v>
       </c>
       <c r="E268" t="s">
         <v>63</v>
@@ -5145,13 +5145,13 @@
         <v>43</v>
       </c>
       <c r="B269">
-        <v>104.9209317049088</v>
+        <v>75.75233835867607</v>
       </c>
       <c r="C269">
-        <v>104.815488544885</v>
+        <v>75.66873904458072</v>
       </c>
       <c r="D269">
-        <v>0.1054431600237251</v>
+        <v>0.08359931409535193</v>
       </c>
       <c r="E269" t="s">
         <v>64</v>
@@ -5162,13 +5162,13 @@
         <v>43</v>
       </c>
       <c r="B270">
-        <v>105.9899624052343</v>
+        <v>101.2638837174825</v>
       </c>
       <c r="C270">
-        <v>105.8701124222063</v>
+        <v>101.1499070695939</v>
       </c>
       <c r="D270">
-        <v>0.1198499830279758</v>
+        <v>0.1139766478886912</v>
       </c>
       <c r="E270" t="s">
         <v>65</v>
@@ -5179,13 +5179,13 @@
         <v>43</v>
       </c>
       <c r="B271">
-        <v>103.3132132430596</v>
+        <v>86.68846734287982</v>
       </c>
       <c r="C271">
-        <v>103.2004943468681</v>
+        <v>86.59192859281353</v>
       </c>
       <c r="D271">
-        <v>0.1127188961914811</v>
+        <v>0.09653875006628709</v>
       </c>
       <c r="E271" t="s">
         <v>66</v>
@@ -5196,13 +5196,13 @@
         <v>43</v>
       </c>
       <c r="B272">
-        <v>106.9721578817352</v>
+        <v>85.81476792395239</v>
       </c>
       <c r="C272">
-        <v>106.8619024607075</v>
+        <v>85.71911959689712</v>
       </c>
       <c r="D272">
-        <v>0.1102554210277304</v>
+        <v>0.09564832705527238</v>
       </c>
       <c r="E272" t="s">
         <v>67</v>
@@ -5213,13 +5213,13 @@
         <v>43</v>
       </c>
       <c r="B273">
-        <v>106.8177712164456</v>
+        <v>81.55065737274444</v>
       </c>
       <c r="C273">
-        <v>106.7097761331666</v>
+        <v>81.4600903610278</v>
       </c>
       <c r="D273">
-        <v>0.1079950832789507</v>
+        <v>0.09056701171664372</v>
       </c>
       <c r="E273" t="s">
         <v>68</v>
@@ -5230,13 +5230,13 @@
         <v>43</v>
       </c>
       <c r="B274">
-        <v>103.675941103797</v>
+        <v>93.93521899761591</v>
       </c>
       <c r="C274">
-        <v>103.55926104372</v>
+        <v>93.83004763642423</v>
       </c>
       <c r="D274">
-        <v>0.1166800600770728</v>
+        <v>0.1051713611916796</v>
       </c>
       <c r="E274" t="s">
         <v>69</v>

</xml_diff>